<commit_message>
braskem: horas por atividade em vez de por etapa (Marcus 8h, Gabriel 38h)
Conforme solicitação do Marcus: stages ficam sem horas, cada
sub-atividade individual recebe suas horas (K=Marcus, L=Gabriel).
Totais inalterados.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0144GG7dJhKbZ5sWAH3QTbQX
</commit_message>
<xml_diff>
--- a/braskem_pe5/Proposta_Braskem_PE5_DEM.xlsx
+++ b/braskem_pe5/Proposta_Braskem_PE5_DEM.xlsx
@@ -2465,12 +2465,6 @@
       <c r="H9" t="n">
         <v>5</v>
       </c>
-      <c r="K9" t="n">
-        <v>2</v>
-      </c>
-      <c r="L9" t="n">
-        <v>8</v>
-      </c>
       <c r="N9" s="141" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1">
@@ -2484,6 +2478,9 @@
       <c r="E10" s="61" t="n"/>
       <c r="F10" s="73" t="n"/>
       <c r="G10" s="56" t="n"/>
+      <c r="L10" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="B11" s="55" t="inlineStr">
@@ -2496,6 +2493,12 @@
       <c r="E11" s="62" t="n"/>
       <c r="F11" s="73" t="n"/>
       <c r="G11" s="56" t="n"/>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="12" ht="15.75" customHeight="1" thickBot="1">
       <c r="B12" s="55" t="inlineStr">
@@ -2508,6 +2511,12 @@
       <c r="E12" s="62" t="n"/>
       <c r="F12" s="73" t="n"/>
       <c r="G12" s="56" t="n"/>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" thickBot="1">
       <c r="B13" s="66" t="inlineStr">
@@ -2525,12 +2534,6 @@
       <c r="G13" s="56" t="n"/>
       <c r="H13" t="n">
         <v>15</v>
-      </c>
-      <c r="K13" t="n">
-        <v>2</v>
-      </c>
-      <c r="L13" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
@@ -2544,6 +2547,9 @@
       <c r="E14" s="73" t="n"/>
       <c r="F14" s="61" t="n"/>
       <c r="G14" s="56" t="n"/>
+      <c r="L14" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="B15" s="55" t="inlineStr">
@@ -2556,6 +2562,9 @@
       <c r="E15" s="73" t="n"/>
       <c r="F15" s="62" t="n"/>
       <c r="G15" s="56" t="n"/>
+      <c r="L15" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" thickBot="1">
       <c r="B16" s="55" t="inlineStr">
@@ -2568,6 +2577,12 @@
       <c r="E16" s="73" t="n"/>
       <c r="F16" s="62" t="n"/>
       <c r="G16" s="56" t="n"/>
+      <c r="K16" t="n">
+        <v>2</v>
+      </c>
+      <c r="L16" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" thickBot="1">
       <c r="B17" s="66" t="inlineStr">
@@ -2586,12 +2601,6 @@
       <c r="H17" t="n">
         <v>5</v>
       </c>
-      <c r="K17" t="n">
-        <v>2</v>
-      </c>
-      <c r="L17" t="n">
-        <v>8</v>
-      </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="B18" s="55" t="inlineStr">
@@ -2604,6 +2613,9 @@
       <c r="E18" s="73" t="n"/>
       <c r="F18" s="73" t="n"/>
       <c r="G18" s="62" t="n"/>
+      <c r="L18" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="B19" s="55" t="inlineStr">
@@ -2616,6 +2628,12 @@
       <c r="E19" s="73" t="n"/>
       <c r="F19" s="73" t="n"/>
       <c r="G19" s="62" t="n"/>
+      <c r="K19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" thickBot="1">
       <c r="B20" s="64" t="inlineStr">
@@ -2628,6 +2646,12 @@
       <c r="E20" s="73" t="n"/>
       <c r="F20" s="73" t="n"/>
       <c r="G20" s="62" t="n"/>
+      <c r="K20" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" thickBot="1">
       <c r="B21" s="66" t="inlineStr">

</xml_diff>

<commit_message>
proposta braskem: remove linhas em branco da aba Proposta
43 linhas vazias removidas do intervalo 18-72 da aba Proposta,
deixando o layout compacto sem espaços desnecessários entre seções.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0144GG7dJhKbZ5sWAH3QTbQX
</commit_message>
<xml_diff>
--- a/braskem_pe5/Proposta_Braskem_PE5_DEM.xlsx
+++ b/braskem_pe5/Proposta_Braskem_PE5_DEM.xlsx
@@ -1630,7 +1630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N73"/>
+  <dimension ref="A1:S30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="12.75"/>
   <cols>
     <col width="2.85546875" customWidth="1" style="1" min="1" max="1"/>
@@ -1872,71 +1872,25 @@
       <c r="I17" s="14" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="123" t="n"/>
-      <c r="C18" s="124" t="n"/>
-      <c r="D18" s="125" t="n"/>
-      <c r="E18" s="125" t="n"/>
-      <c r="F18" s="125" t="n"/>
-      <c r="G18" s="125" t="n"/>
+      <c r="B18" s="128" t="inlineStr">
+        <is>
+          <t>Objetivo: Identificar as causas e propor mitigações para o embuchamento (clogging) de pó de PEAD na rosca transportadora da unidade PE5 (RS), utilizando simulação pelo Método de Elementos Discretos (DEM) no Star-CCM+ 2506. Serão avaliados dois cenários: rosca de pá helicoidal contínua (padrão) e rosca cut-flight, com foco nas zonas de velocidade de partícula próxima a zero, indicativas de embuchamento.</t>
+        </is>
+      </c>
+      <c r="G18" s="124" t="n"/>
       <c r="I18" s="14" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="20" t="n"/>
-      <c r="C19" s="21" t="n"/>
-      <c r="D19" s="111" t="n"/>
-      <c r="E19" s="23" t="n"/>
-      <c r="F19" s="126" t="n"/>
-      <c r="G19" s="127" t="n"/>
+      <c r="B19" s="128" t="inlineStr">
+        <is>
+          <t>Recursos: Empregaremos neste projeto uma equipe técnica de consultores experientes na solução de problemas industriais com o apoio de ferramentas de CAE avançadas da SIEMENS, como o STAR-CCM+, referência mundial na área de fluidodinâmica.</t>
+        </is>
+      </c>
+      <c r="G19" s="124" t="n"/>
       <c r="I19" s="14" t="n"/>
     </row>
     <row r="20" ht="13.9" customHeight="1">
       <c r="B20" s="128" t="inlineStr">
-        <is>
-          <t>Objetivo: Identificar as causas e propor mitigações para o embuchamento (clogging) de pó de PEAD na rosca transportadora da unidade PE5 (RS), utilizando simulação pelo Método de Elementos Discretos (DEM) no Star-CCM+ 2506. Serão avaliados dois cenários: rosca de pá helicoidal contínua (padrão) e rosca cut-flight, com foco nas zonas de velocidade de partícula próxima a zero, indicativas de embuchamento.</t>
-        </is>
-      </c>
-      <c r="G20" s="124" t="n"/>
-      <c r="I20" s="14" t="n"/>
-    </row>
-    <row r="21" ht="13.9" customHeight="1">
-      <c r="B21" s="82" t="n"/>
-      <c r="G21" s="124" t="n"/>
-      <c r="I21" s="14" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="82" t="n"/>
-      <c r="C22" s="26" t="n"/>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="129" t="n"/>
-      <c r="G22" s="130" t="n"/>
-      <c r="I22" s="14" t="n"/>
-    </row>
-    <row r="23" ht="12.75" customHeight="1">
-      <c r="B23" s="128" t="inlineStr">
-        <is>
-          <t>Recursos: Empregaremos neste projeto uma equipe técnica de consultores experientes na solução de problemas industriais com o apoio de ferramentas de CAE avançadas da SIEMENS, como o STAR-CCM+, referência mundial na área de fluidodinâmica.</t>
-        </is>
-      </c>
-      <c r="G23" s="124" t="n"/>
-      <c r="I23" s="14" t="n"/>
-    </row>
-    <row r="24" ht="12.75" customHeight="1">
-      <c r="B24" s="82" t="n"/>
-      <c r="G24" s="124" t="n"/>
-      <c r="I24" s="14" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="36" t="n"/>
-      <c r="C25" s="26" t="n"/>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
-      <c r="F25" s="129" t="n"/>
-      <c r="G25" s="130" t="n"/>
-      <c r="I25" s="14" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="128" t="inlineStr">
         <is>
           <t>Escopo: A CAEXPERTS desenvolverá o estudo em 4 etapas, descritas a seguir:
 Na Etapa 1 (Configuração Inicial — 5 dias): Ajuste da geometria 3D da rosca com os parâmetros reais fornecidos pela Braskem (D_screw, D_shaft, pitch, RPM); configuração do domínio DEM no Star-CCM+ 2506 com física de contato Hertz-Mindlin e Liquid Bridge Force (Lian, 1993) para modelar a coesão hexano-PEAD; calibração dos parâmetros de partícula com base na granulometria do PEAD fornecida.
@@ -1945,277 +1899,118 @@
 Na Etapa 4 (Reunião Final Online — dia 25): Apresentação dos resultados e recomendações de mitigação do embuchamento à equipe técnica da Braskem PE5.</t>
         </is>
       </c>
-      <c r="G26" s="124" t="n"/>
-      <c r="I26" s="14" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="82" t="n"/>
-      <c r="G27" s="124" t="n"/>
-      <c r="I27" s="14" t="n"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="82" t="n"/>
-      <c r="G28" s="124" t="n"/>
-      <c r="I28" s="14" t="n"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="82" t="n"/>
-      <c r="G29" s="124" t="n"/>
-      <c r="I29" s="14" t="n"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="82" t="n"/>
-      <c r="G30" s="124" t="n"/>
-      <c r="I30" s="14" t="n"/>
-    </row>
-    <row r="31">
-      <c r="B31" s="82" t="n"/>
-      <c r="G31" s="124" t="n"/>
-      <c r="I31" s="14" t="n"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="82" t="n"/>
-      <c r="G32" s="124" t="n"/>
-      <c r="I32" s="14" t="n"/>
-    </row>
-    <row r="33">
-      <c r="B33" s="82" t="n"/>
-      <c r="G33" s="124" t="n"/>
-      <c r="I33" s="14" t="n"/>
-    </row>
-    <row r="34">
-      <c r="B34" s="82" t="n"/>
-      <c r="G34" s="124" t="n"/>
-      <c r="I34" s="14" t="n"/>
-    </row>
-    <row r="35">
-      <c r="B35" s="82" t="n"/>
-      <c r="G35" s="124" t="n"/>
-      <c r="I35" s="14" t="n"/>
-    </row>
-    <row r="36">
-      <c r="B36" s="82" t="n"/>
-      <c r="G36" s="124" t="n"/>
-      <c r="I36" s="14" t="n"/>
-    </row>
-    <row r="37">
-      <c r="B37" s="82" t="n"/>
-      <c r="G37" s="124" t="n"/>
-      <c r="I37" s="14" t="n"/>
-    </row>
-    <row r="38">
-      <c r="B38" s="82" t="n"/>
-      <c r="G38" s="124" t="n"/>
-      <c r="I38" s="14" t="n"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="82" t="n"/>
-      <c r="G39" s="124" t="n"/>
-      <c r="I39" s="14" t="n"/>
-    </row>
-    <row r="40">
-      <c r="B40" s="82" t="n"/>
-      <c r="G40" s="124" t="n"/>
-      <c r="I40" s="14" t="n"/>
-    </row>
-    <row r="41">
-      <c r="B41" s="82" t="n"/>
-      <c r="G41" s="124" t="n"/>
-      <c r="I41" s="14" t="n"/>
-    </row>
-    <row r="42">
-      <c r="B42" s="43" t="n"/>
-      <c r="C42" s="83" t="n"/>
-      <c r="D42" s="83" t="n"/>
-      <c r="E42" s="83" t="n"/>
-      <c r="F42" s="83" t="n"/>
-      <c r="G42" s="44" t="n"/>
-      <c r="I42" s="14" t="n"/>
-    </row>
-    <row r="43" ht="12.75" customHeight="1">
-      <c r="B43" s="128" t="inlineStr">
+      <c r="G20" s="124" t="n"/>
+      <c r="I20" s="14" t="n"/>
+    </row>
+    <row r="21" ht="13.9" customHeight="1">
+      <c r="B21" s="128" t="inlineStr">
         <is>
           <t>Cronograma de Atividades: A execução do projeto está prevista para ser realizada em 25 dias, conforme cronograma de atividades em anexo. A primeira etapa se iniciará oficialmente a partir do dia subsequente ao recebimento dos documentos com os dados necessários ao projeto. Cada etapa está com a duração em dias prevista conforme indicado abaixo:
 Etapa 1: 5 dias;   Etapa 2: 15 dias;   Etapa 3: 5 dias;   Reunião Final: dia 25.</t>
         </is>
       </c>
-      <c r="G43" s="124" t="n"/>
-      <c r="I43" s="14" t="n"/>
-    </row>
-    <row r="44" ht="12.75" customHeight="1">
-      <c r="B44" s="82" t="n"/>
-      <c r="G44" s="124" t="n"/>
-      <c r="I44" s="14" t="n"/>
-    </row>
-    <row r="45" ht="12.75" customHeight="1">
-      <c r="B45" s="82" t="n"/>
-      <c r="G45" s="124" t="n"/>
-      <c r="I45" s="14" t="n"/>
-    </row>
-    <row r="46" ht="12.75" customHeight="1">
-      <c r="B46" s="82" t="n"/>
-      <c r="G46" s="124" t="n"/>
-      <c r="I46" s="14" t="n"/>
-    </row>
-    <row r="47">
-      <c r="B47" s="82" t="n"/>
-      <c r="G47" s="124" t="n"/>
-      <c r="I47" s="14" t="n"/>
-    </row>
-    <row r="48">
-      <c r="B48" s="85" t="n"/>
-      <c r="C48" s="86" t="n"/>
-      <c r="D48" s="86" t="n"/>
-      <c r="E48" s="86" t="n"/>
-      <c r="F48" s="86" t="n"/>
-      <c r="G48" s="87" t="n"/>
-      <c r="I48" s="14" t="n"/>
-    </row>
-    <row r="49" ht="13.9" customHeight="1">
-      <c r="B49" s="128" t="inlineStr">
+      <c r="G21" s="124" t="n"/>
+      <c r="I21" s="14" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="128" t="inlineStr">
         <is>
           <t>Requisitos/Dados Necessários ao Projeto: Diâmetro externo da pá (D_screw, mm), diâmetro do eixo (D_shaft, mm), passo da hélice (pitch, mm) e RPM de operação; granulometria do pó de PEAD (D10, D50, D90) — alternativamente, confirmação de semelhança com pó de talco; densidade aparente do PEAD (bulk density, kg/m³); localização típica do embuchamento (início/meio/fim da rosca); tipo de rosca em operação (padrão ou cut-flight); e, se disponível, desenho técnico ou croqui com cotas e fotos do equipamento.</t>
         </is>
       </c>
-      <c r="G49" s="124" t="n"/>
-      <c r="I49" s="14" t="n"/>
-    </row>
-    <row r="50">
-      <c r="B50" s="82" t="n"/>
-      <c r="G50" s="124" t="n"/>
-      <c r="I50" s="14" t="n"/>
-    </row>
-    <row r="51">
-      <c r="B51" s="85" t="n"/>
-      <c r="C51" s="86" t="n"/>
-      <c r="D51" s="86" t="n"/>
-      <c r="E51" s="86" t="n"/>
-      <c r="F51" s="86" t="n"/>
-      <c r="G51" s="87" t="n"/>
-      <c r="I51" s="14" t="n"/>
-    </row>
-    <row r="52" ht="13.9" customHeight="1">
-      <c r="B52" s="128" t="inlineStr">
+      <c r="G22" s="124" t="n"/>
+      <c r="I22" s="14" t="n"/>
+    </row>
+    <row r="23" ht="12.75" customHeight="1">
+      <c r="B23" s="128" t="inlineStr">
         <is>
           <t>Entregáveis do Projeto: Relatório técnico em formato .ppt contendo: geometria 3D da rosca simulada (arquivo STEP), campos de velocidade e distribuição de partículas DEM, identificação das zonas de embuchamento, comparação quantitativa entre rosca padrão e cut-flight, e recomendações de mitigação fundamentadas nos resultados das simulações.</t>
         </is>
       </c>
-      <c r="G52" s="124" t="n"/>
-      <c r="I52" s="14" t="n"/>
-    </row>
-    <row r="53">
-      <c r="B53" s="85" t="n"/>
-      <c r="C53" s="86" t="n"/>
-      <c r="D53" s="7" t="n"/>
-      <c r="E53" s="7" t="n"/>
-      <c r="F53" s="129" t="n"/>
-      <c r="G53" s="130" t="n"/>
-      <c r="I53" s="14" t="n"/>
-    </row>
-    <row r="54" ht="13.9" customHeight="1">
-      <c r="B54" s="128" t="inlineStr">
+      <c r="G23" s="124" t="n"/>
+      <c r="I23" s="14" t="n"/>
+    </row>
+    <row r="24" ht="12.75" customHeight="1">
+      <c r="B24" s="128" t="inlineStr">
         <is>
           <t>Quem Somos: A CAEXPERTS é uma empresa especializada em digitalização da engenharia que conta com uma rede de consultores pioneiros da implantação de tecnologias de simulação computacional na indústria nacional. Somos parceiros tecnológicos da SIEMENS Digital Industries Software, onde contamos com um portifólio de ferramentas de CAE mais completo do mercado.</t>
         </is>
       </c>
-      <c r="G54" s="124" t="n"/>
-      <c r="I54" s="14" t="n"/>
-    </row>
-    <row r="55" ht="13.9" customHeight="1">
-      <c r="B55" s="82" t="n"/>
-      <c r="G55" s="124" t="n"/>
-      <c r="I55" s="14" t="n"/>
-    </row>
-    <row r="56" ht="12.75" customHeight="1">
-      <c r="B56" s="82" t="n"/>
-      <c r="G56" s="124" t="n"/>
-      <c r="I56" s="14" t="n"/>
-    </row>
-    <row r="57">
-      <c r="B57" s="39" t="n"/>
-      <c r="C57" s="40" t="n"/>
-      <c r="D57" s="40" t="n"/>
-      <c r="E57" s="40" t="n"/>
-      <c r="F57" s="40" t="n"/>
-      <c r="G57" s="41" t="n"/>
-      <c r="I57" s="14" t="n"/>
-    </row>
-    <row r="58" ht="15.75" customHeight="1">
-      <c r="B58" s="91" t="inlineStr">
+      <c r="G24" s="124" t="n"/>
+      <c r="I24" s="14" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="91" t="inlineStr">
         <is>
           <t>INVESTIMENTO TOTAL</t>
         </is>
       </c>
-      <c r="C58" s="131" t="n"/>
-      <c r="D58" s="131" t="n"/>
-      <c r="E58" s="131" t="n"/>
-      <c r="F58" s="132">
+      <c r="C25" s="131" t="n"/>
+      <c r="D25" s="131" t="n"/>
+      <c r="E25" s="131" t="n"/>
+      <c r="F25" s="132">
         <f>G17</f>
         <v/>
       </c>
-      <c r="G58" s="133" t="n"/>
-      <c r="I58" s="14" t="n"/>
-    </row>
-    <row r="59">
-      <c r="B59" s="9" t="n"/>
-      <c r="C59" s="26" t="n"/>
-      <c r="D59" s="8" t="n"/>
-      <c r="E59" s="27" t="n"/>
-      <c r="F59" s="27" t="n"/>
-      <c r="G59" s="134" t="n"/>
-      <c r="I59" s="14" t="n"/>
-    </row>
-    <row r="60">
-      <c r="B60" s="34" t="inlineStr">
+      <c r="G25" s="133" t="n"/>
+      <c r="I25" s="14" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="34" t="inlineStr">
         <is>
           <t>Observações:</t>
         </is>
       </c>
-      <c r="C60" s="15" t="n"/>
-      <c r="D60" s="16" t="n"/>
-      <c r="I60" s="14" t="n"/>
-    </row>
-    <row r="61">
-      <c r="B61" s="96" t="inlineStr">
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="16" t="n"/>
+      <c r="I26" s="14" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="96" t="inlineStr">
         <is>
           <t>Condições de Pagamento: 30 dias.</t>
         </is>
       </c>
-      <c r="I61" s="14" t="n"/>
-    </row>
-    <row r="62">
-      <c r="B62" s="96" t="inlineStr">
+      <c r="I27" s="14" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="96" t="inlineStr">
         <is>
           <t>Faturamento: Nota fiscal de serviços</t>
         </is>
       </c>
-      <c r="I62" s="14" t="n"/>
-    </row>
-    <row r="64">
-      <c r="B64" s="135" t="inlineStr">
+      <c r="I28" s="14" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="135" t="inlineStr">
         <is>
           <t>Aceitação desta proposta via emissão de pedido de compras ou contrato específico</t>
         </is>
       </c>
-      <c r="C64" s="136" t="n"/>
-      <c r="D64" s="136" t="n"/>
-      <c r="E64" s="136" t="n"/>
-      <c r="F64" s="136" t="n"/>
-      <c r="G64" s="137" t="n"/>
-    </row>
-    <row r="67">
-      <c r="H67" s="17" t="n"/>
-    </row>
-    <row r="68">
-      <c r="H68" s="17" t="n"/>
-    </row>
-    <row r="73" ht="23.25" customHeight="1">
-      <c r="B73" s="88" t="inlineStr">
+      <c r="C29" s="136" t="n"/>
+      <c r="D29" s="136" t="n"/>
+      <c r="E29" s="136" t="n"/>
+      <c r="F29" s="136" t="n"/>
+      <c r="G29" s="137" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="88" t="inlineStr">
         <is>
           <t>ANEXO - CRONOGRAMA DE ATIVIDADES</t>
         </is>
       </c>
     </row>
+    <row r="43" ht="12.75" customHeight="1"/>
+    <row r="44" ht="12.75" customHeight="1"/>
+    <row r="45" ht="12.75" customHeight="1"/>
+    <row r="46" ht="12.75" customHeight="1"/>
+    <row r="49" ht="13.9" customHeight="1"/>
+    <row r="52" ht="13.9" customHeight="1"/>
+    <row r="54" ht="13.9" customHeight="1"/>
+    <row r="55" ht="13.9" customHeight="1"/>
+    <row r="56" ht="12.75" customHeight="1"/>
+    <row r="58" ht="15.75" customHeight="1"/>
+    <row r="73" ht="23.25" customHeight="1"/>
   </sheetData>
   <mergeCells count="29">
     <mergeCell ref="E10:G10"/>

</xml_diff>

<commit_message>
proposta braskem: compacta aba Proposta (max 1 linha em branco entre seções)
Reduz de 73 para 40 linhas: qualquer sequência de N≥2 linhas vazias
vira exatamente 1 linha vazia. Conteúdo intacto (Objetivo, Escopo,
Cronograma, Requisitos, Entregáveis, Quem Somos, Investimento, Anexo).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0144GG7dJhKbZ5sWAH3QTbQX
</commit_message>
<xml_diff>
--- a/braskem_pe5/Proposta_Braskem_PE5_DEM.xlsx
+++ b/braskem_pe5/Proposta_Braskem_PE5_DEM.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposta" sheetId="1" state="visible" r:id="rId1"/>
@@ -20,15 +20,23 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -51,11 +59,6 @@
       <color rgb="FF3F3F3F"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -207,6 +210,12 @@
       <sz val="10"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color rgb="FF0000FF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -251,7 +260,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="43">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -295,19 +304,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color rgb="FF3F3F3F"/>
@@ -354,30 +350,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color rgb="FF3F3F3F"/>
@@ -418,17 +390,6 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -667,26 +628,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -707,15 +648,6 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -739,21 +671,61 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="11">
+  <cellStyleXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3"/>
     <xf numFmtId="44" fontId="23" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="23" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="23" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="23" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3"/>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="167" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="167" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="143">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -805,7 +777,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -817,7 +789,7 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
@@ -840,9 +812,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
@@ -851,34 +820,34 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -891,66 +860,63 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" pivotButton="0" quotePrefix="0" xfId="7"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" pivotButton="0" quotePrefix="0" xfId="7"/>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" pivotButton="0" quotePrefix="0" xfId="7"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="18" pivotButton="0" quotePrefix="0" xfId="7"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" pivotButton="0" quotePrefix="0" xfId="7"/>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" pivotButton="0" quotePrefix="0" xfId="7"/>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="30" pivotButton="0" quotePrefix="0" xfId="7"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="31" pivotButton="0" quotePrefix="0" xfId="7"/>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="26" pivotButton="0" quotePrefix="0" xfId="7"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="27" pivotButton="0" quotePrefix="0" xfId="7"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="23" pivotButton="0" quotePrefix="0" xfId="7"/>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" pivotButton="0" quotePrefix="0" xfId="7"/>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="29" pivotButton="0" quotePrefix="0" xfId="7"/>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="25" pivotButton="0" quotePrefix="0" xfId="7"/>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="32" pivotButton="0" quotePrefix="1" xfId="7"/>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="28" pivotButton="0" quotePrefix="1" xfId="7"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="7">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="7"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="7"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="10"/>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
@@ -963,156 +929,91 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="10">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="24" fillId="5" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="5" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="24" fillId="5" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="24" fillId="5" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="10"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="17">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="16">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="21">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="21">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="11">
+  <cellStyles count="22">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Saída" xfId="1" builtinId="21"/>
     <cellStyle name="Moeda" xfId="2" builtinId="4"/>
@@ -1124,6 +1025,17 @@
     <cellStyle name="Moeda 2" xfId="8"/>
     <cellStyle name="Porcentagem 3" xfId="9"/>
     <cellStyle name="Porcentagem" xfId="10" builtinId="5"/>
+    <cellStyle name="Saída 2" xfId="11"/>
+    <cellStyle name="Moeda 3" xfId="12"/>
+    <cellStyle name="Vírgula 3" xfId="13"/>
+    <cellStyle name="Porcentagem 2 2" xfId="14"/>
+    <cellStyle name="Vírgula 2 2" xfId="15"/>
+    <cellStyle name="Hiperlink 2" xfId="16"/>
+    <cellStyle name="Normal 2 2" xfId="17"/>
+    <cellStyle name="Moeda 2 2" xfId="18"/>
+    <cellStyle name="Porcentagem 3 2" xfId="19"/>
+    <cellStyle name="Porcentagem 4" xfId="20"/>
+    <cellStyle name="Normal 3" xfId="21"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors/>
@@ -1142,8 +1054,8 @@
     <to>
       <col>9</col>
       <colOff>0</colOff>
-      <row>59</row>
-      <rowOff>142875</rowOff>
+      <row>56</row>
+      <rowOff>57150</rowOff>
     </to>
     <pic>
       <nvPicPr>
@@ -1185,8 +1097,8 @@
     <to>
       <col>9</col>
       <colOff>0</colOff>
-      <row>59</row>
-      <rowOff>142875</rowOff>
+      <row>56</row>
+      <rowOff>57150</rowOff>
     </to>
     <pic>
       <nvPicPr>
@@ -1630,26 +1542,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S30"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="12.75"/>
   <cols>
-    <col width="2.85546875" customWidth="1" style="1" min="1" max="1"/>
-    <col width="65.7109375" customWidth="1" style="1" min="2" max="2"/>
-    <col width="18.85546875" customWidth="1" style="1" min="3" max="3"/>
-    <col width="10.85546875" customWidth="1" style="6" min="4" max="4"/>
-    <col width="8.42578125" customWidth="1" style="1" min="5" max="5"/>
-    <col width="12.5703125" customWidth="1" style="1" min="6" max="7"/>
-    <col hidden="1" width="12.42578125" customWidth="1" style="1" min="8" max="8"/>
-    <col width="4.140625" customWidth="1" style="1" min="9" max="9"/>
-    <col hidden="1" width="11.28515625" customWidth="1" style="1" min="10" max="10"/>
-    <col hidden="1" width="37" customWidth="1" style="1" min="11" max="11"/>
-    <col hidden="1" width="10.42578125" customWidth="1" style="1" min="12" max="12"/>
-    <col hidden="1" width="7.42578125" customWidth="1" style="1" min="13" max="13"/>
-    <col hidden="1" width="11.42578125" customWidth="1" style="116" min="14" max="14"/>
-    <col hidden="1" width="8.85546875" customWidth="1" style="1" min="15" max="16384"/>
+    <col width="2.85546875" customWidth="1" style="89" min="1" max="1"/>
+    <col width="65.7109375" customWidth="1" style="89" min="2" max="2"/>
+    <col width="18.85546875" customWidth="1" style="89" min="3" max="3"/>
+    <col width="10.85546875" customWidth="1" style="90" min="4" max="4"/>
+    <col width="8.42578125" customWidth="1" style="89" min="5" max="5"/>
+    <col width="12.5703125" customWidth="1" style="89" min="6" max="7"/>
+    <col hidden="1" width="12.42578125" customWidth="1" style="89" min="8" max="8"/>
+    <col width="4.140625" customWidth="1" style="89" min="9" max="9"/>
+    <col hidden="1" width="11.28515625" customWidth="1" style="89" min="10" max="10"/>
+    <col hidden="1" width="37" customWidth="1" style="89" min="11" max="11"/>
+    <col hidden="1" width="10.42578125" customWidth="1" style="89" min="12" max="12"/>
+    <col hidden="1" width="7.42578125" customWidth="1" style="89" min="13" max="13"/>
+    <col hidden="1" width="11.42578125" customWidth="1" style="19" min="14" max="14"/>
+    <col hidden="1" width="8.85546875" customWidth="1" style="89" min="15" max="15"/>
+    <col hidden="1" width="8.85546875" customWidth="1" style="89" min="16" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" customHeight="1">
+    <row r="1" ht="21" customHeight="1" s="117">
       <c r="B1" s="29" t="n"/>
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="3" t="n"/>
@@ -1658,7 +1571,7 @@
       <c r="G1" s="2" t="n"/>
       <c r="H1" s="2" t="n"/>
     </row>
-    <row r="2" ht="21" customHeight="1">
+    <row r="2" ht="21" customHeight="1" s="117">
       <c r="B2" s="4" t="n"/>
       <c r="C2" s="5" t="n"/>
       <c r="D2" s="30" t="inlineStr">
@@ -1666,63 +1579,63 @@
           <t>DATA:</t>
         </is>
       </c>
-      <c r="E2" s="98" t="n">
+      <c r="E2" s="94" t="n">
         <v>46196</v>
       </c>
     </row>
-    <row r="3" ht="12.95" customHeight="1">
+    <row r="3" ht="12.95" customHeight="1" s="117">
       <c r="C3" s="7" t="n"/>
       <c r="D3" s="8" t="n"/>
     </row>
-    <row r="4" ht="12.95" customHeight="1">
+    <row r="4" ht="12.95" customHeight="1" s="117">
       <c r="C4" s="4" t="n"/>
       <c r="D4" s="30" t="inlineStr">
         <is>
           <t>DE:</t>
         </is>
       </c>
-      <c r="E4" s="99" t="inlineStr">
-        <is>
-          <t>Gabriel Hernandez Rozo</t>
-        </is>
-      </c>
-      <c r="K4" s="9" t="n"/>
-      <c r="L4" s="9" t="n"/>
-      <c r="M4" s="9" t="n"/>
-      <c r="N4" s="117" t="n"/>
-    </row>
-    <row r="5" ht="12.95" customFormat="1" customHeight="1" s="9">
-      <c r="A5" s="1" t="n"/>
+      <c r="E4" s="116" t="inlineStr">
+        <is>
+          <t>Ricardo Barbosa de Barros</t>
+        </is>
+      </c>
+      <c r="K4" s="83" t="n"/>
+      <c r="L4" s="83" t="n"/>
+      <c r="M4" s="83" t="n"/>
+      <c r="N4" s="18" t="n"/>
+    </row>
+    <row r="5" ht="12.95" customFormat="1" customHeight="1" s="83">
+      <c r="A5" s="89" t="n"/>
       <c r="C5" s="4" t="n"/>
       <c r="D5" s="31" t="n"/>
-      <c r="E5" s="33" t="inlineStr">
-        <is>
-          <t>ghrozo97@gmail.com</t>
-        </is>
-      </c>
-      <c r="F5" s="33" t="n"/>
-      <c r="G5" s="33" t="n"/>
-      <c r="N5" s="117" t="n"/>
-    </row>
-    <row r="6" ht="12.95" customFormat="1" customHeight="1" s="9">
-      <c r="A6" s="1" t="n"/>
+      <c r="E5" s="118" t="inlineStr">
+        <is>
+          <t>(48) 9 9919 3243</t>
+        </is>
+      </c>
+      <c r="F5" s="118" t="n"/>
+      <c r="G5" s="118" t="n"/>
+      <c r="N5" s="18" t="n"/>
+    </row>
+    <row r="6" ht="12.95" customFormat="1" customHeight="1" s="83">
+      <c r="A6" s="89" t="n"/>
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="4" t="n"/>
-      <c r="E6" s="97" t="inlineStr">
-        <is>
-          <t>CAExperts — Florianópolis/SC</t>
-        </is>
-      </c>
-      <c r="N6" s="117" t="n"/>
-    </row>
-    <row r="7" ht="12.95" customFormat="1" customHeight="1" s="9">
-      <c r="A7" s="1" t="n"/>
+      <c r="E6" s="115" t="inlineStr">
+        <is>
+          <t>barros@caexperts.com.br</t>
+        </is>
+      </c>
+      <c r="N6" s="18" t="n"/>
+    </row>
+    <row r="7" ht="12.95" customFormat="1" customHeight="1" s="83">
+      <c r="A7" s="89" t="n"/>
       <c r="C7" s="4" t="n"/>
-      <c r="E7" s="97" t="n"/>
-      <c r="N7" s="117" t="n"/>
-    </row>
-    <row r="8" ht="12.95" customFormat="1" customHeight="1" s="9">
-      <c r="A8" s="1" t="n"/>
+      <c r="E7" s="98" t="n"/>
+      <c r="N7" s="18" t="n"/>
+    </row>
+    <row r="8" ht="12.95" customFormat="1" customHeight="1" s="83">
+      <c r="A8" s="89" t="n"/>
       <c r="B8" s="29" t="inlineStr">
         <is>
           <t>Razão Social: Creative Solutions Engenharia e Consultoria LTDA</t>
@@ -1734,15 +1647,15 @@
           <t>PARA:</t>
         </is>
       </c>
-      <c r="E8" s="100" t="inlineStr">
+      <c r="E8" s="110" t="inlineStr">
         <is>
           <t>Braskem S.A. — Unidade PE5 (RS)</t>
         </is>
       </c>
-      <c r="N8" s="117" t="n"/>
-    </row>
-    <row r="9" ht="12.95" customFormat="1" customHeight="1" s="9">
-      <c r="A9" s="1" t="n"/>
+      <c r="N8" s="18" t="n"/>
+    </row>
+    <row r="9" ht="12.95" customFormat="1" customHeight="1" s="83">
+      <c r="A9" s="89" t="n"/>
       <c r="B9" s="29" t="inlineStr">
         <is>
           <t>CNPJ: 15.806.919/0001-44 - Inscrição Estadual: 25.676.225-2</t>
@@ -1750,15 +1663,15 @@
       </c>
       <c r="C9" s="4" t="n"/>
       <c r="D9" s="4" t="n"/>
-      <c r="E9" s="101" t="inlineStr">
+      <c r="E9" s="96" t="inlineStr">
         <is>
           <t>Jeferson Diefenthaler</t>
         </is>
       </c>
-      <c r="N9" s="117" t="n"/>
-    </row>
-    <row r="10" ht="12.95" customFormat="1" customHeight="1" s="9">
-      <c r="A10" s="1" t="n"/>
+      <c r="N9" s="18" t="n"/>
+    </row>
+    <row r="10" ht="12.95" customFormat="1" customHeight="1" s="83">
+      <c r="A10" s="89" t="n"/>
       <c r="B10" s="29" t="inlineStr">
         <is>
           <t>Rod Jose Carlos Daux, km 01 - Edifício CELTA, 3º andar - Sala 2.02</t>
@@ -1766,11 +1679,15 @@
       </c>
       <c r="C10" s="4" t="n"/>
       <c r="D10" s="4" t="n"/>
-      <c r="E10" s="102" t="inlineStr"/>
-      <c r="N10" s="117" t="n"/>
-    </row>
-    <row r="11" ht="12.95" customFormat="1" customHeight="1" s="9">
-      <c r="A11" s="1" t="n"/>
+      <c r="E10" s="119" t="inlineStr">
+        <is>
+          <t>jeferson.diefenthaler@braskem.com</t>
+        </is>
+      </c>
+      <c r="N10" s="18" t="n"/>
+    </row>
+    <row r="11" ht="12.95" customFormat="1" customHeight="1" s="83">
+      <c r="A11" s="89" t="n"/>
       <c r="B11" s="29" t="inlineStr">
         <is>
           <t>CEP: 88030-902 - Bairro João Paulo</t>
@@ -1778,11 +1695,11 @@
       </c>
       <c r="C11" s="4" t="n"/>
       <c r="D11" s="4" t="n"/>
-      <c r="E11" s="97" t="inlineStr"/>
-      <c r="N11" s="117" t="n"/>
-    </row>
-    <row r="12" ht="12.95" customFormat="1" customHeight="1" s="9">
-      <c r="A12" s="1" t="n"/>
+      <c r="E11" s="98" t="n"/>
+      <c r="N11" s="18" t="n"/>
+    </row>
+    <row r="12" ht="12.95" customFormat="1" customHeight="1" s="83">
+      <c r="A12" s="89" t="n"/>
       <c r="B12" s="29" t="inlineStr">
         <is>
           <t>Florianópolis – SC – Brasil</t>
@@ -1790,107 +1707,119 @@
       </c>
       <c r="C12" s="4" t="n"/>
       <c r="D12" s="4" t="n"/>
-      <c r="N12" s="117" t="n"/>
-    </row>
-    <row r="13" ht="12.95" customFormat="1" customHeight="1" s="9">
-      <c r="A13" s="1" t="n"/>
+      <c r="N12" s="18" t="n"/>
+    </row>
+    <row r="13" ht="12.95" customFormat="1" customHeight="1" s="83">
+      <c r="A13" s="89" t="n"/>
       <c r="C13" s="4" t="n"/>
       <c r="D13" s="32" t="inlineStr">
         <is>
           <t>VÁLIDO ATÉ:</t>
         </is>
       </c>
-      <c r="E13" s="98">
+      <c r="E13" s="94">
         <f>E2+30</f>
         <v/>
       </c>
-      <c r="N13" s="117" t="n"/>
-    </row>
-    <row r="14" ht="12.95" customHeight="1">
+      <c r="N13" s="18" t="n"/>
+    </row>
+    <row r="14" ht="12.95" customHeight="1" s="117">
       <c r="B14" s="10" t="n"/>
       <c r="C14" s="11" t="n"/>
     </row>
-    <row r="15" ht="21" customHeight="1">
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="12" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="103" t="n"/>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="B16" s="118" t="inlineStr">
+    <row r="15" ht="21" customHeight="1" s="117">
+      <c r="B15" s="86" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C16" s="119" t="n"/>
-      <c r="D16" s="76" t="inlineStr">
+      <c r="C15" s="87" t="n"/>
+      <c r="D15" s="74" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="E16" s="77" t="inlineStr">
+      <c r="E15" s="75" t="inlineStr">
         <is>
           <t>Quant.</t>
         </is>
       </c>
-      <c r="F16" s="78" t="inlineStr">
+      <c r="F15" s="76" t="inlineStr">
         <is>
           <t>Valor Unit.</t>
         </is>
       </c>
-      <c r="G16" s="78" t="inlineStr">
+      <c r="G15" s="76" t="inlineStr">
         <is>
           <t>Valor Total</t>
         </is>
       </c>
-      <c r="I16" s="13" t="n"/>
-    </row>
-    <row r="17" ht="12.75" customHeight="1">
-      <c r="B17" s="120" t="inlineStr">
+      <c r="I15" s="13" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="117">
+      <c r="B16" s="107" t="inlineStr">
         <is>
           <t>Estudo de Embuchamento em Rosca Transportadora — Simulação DEM (PEAD + Hexano)</t>
         </is>
       </c>
-      <c r="C17" s="121" t="n"/>
-      <c r="D17" s="110" t="inlineStr">
+      <c r="C16" s="108" t="n"/>
+      <c r="D16" s="84" t="inlineStr">
         <is>
           <t>Serviço</t>
         </is>
       </c>
-      <c r="E17" s="110" t="n">
+      <c r="E16" s="84" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="122">
+      <c r="F16" s="93">
         <f>ROUND(Cronograma!O5,0)*1.1</f>
         <v/>
       </c>
-      <c r="G17" s="122">
+      <c r="G16" s="93">
         <f>F17</f>
         <v/>
       </c>
+      <c r="I16" s="14" t="n"/>
+    </row>
+    <row r="17" ht="12.75" customHeight="1" s="117">
+      <c r="B17" s="109" t="n"/>
+      <c r="C17" s="91" t="n"/>
+      <c r="D17" s="85" t="n"/>
+      <c r="E17" s="85" t="n"/>
+      <c r="F17" s="85" t="n"/>
+      <c r="G17" s="85" t="n"/>
       <c r="I17" s="14" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="128" t="inlineStr">
-        <is>
-          <t>Objetivo: Identificar as causas e propor mitigações para o embuchamento (clogging) de pó de PEAD na rosca transportadora da unidade PE5 (RS), utilizando simulação pelo Método de Elementos Discretos (DEM) no Star-CCM+ 2506. Serão avaliados dois cenários: rosca de pá helicoidal contínua (padrão) e rosca cut-flight, com foco nas zonas de velocidade de partícula próxima a zero, indicativas de embuchamento.</t>
-        </is>
-      </c>
-      <c r="G18" s="124" t="n"/>
+      <c r="B18" s="88" t="inlineStr">
+        <is>
+          <t>Objetivo: Identificar as causas e propor mitigações para o embuchamento (clogging) de pó de PEAD na rosca transportadora da unidade PE5 (RS), utilizando simulação pelo Método de Elementos Discretos (DEM) no Star-CCM+. Serão avaliados dois cenários: rosca de pá helicoidal contínua (padrão) e rosca cut-flight, com foco nas zonas de velocidade de partícula próxima a zero, indicativas de embuchamento.</t>
+        </is>
+      </c>
+      <c r="G18" s="91" t="n"/>
       <c r="I18" s="14" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="128" t="inlineStr">
+      <c r="B19" s="92" t="n"/>
+      <c r="G19" s="91" t="n"/>
+      <c r="I19" s="14" t="n"/>
+    </row>
+    <row r="20" ht="13.9" customHeight="1" s="117">
+      <c r="B20" s="88" t="inlineStr">
         <is>
           <t>Recursos: Empregaremos neste projeto uma equipe técnica de consultores experientes na solução de problemas industriais com o apoio de ferramentas de CAE avançadas da SIEMENS, como o STAR-CCM+, referência mundial na área de fluidodinâmica.</t>
         </is>
       </c>
-      <c r="G19" s="124" t="n"/>
-      <c r="I19" s="14" t="n"/>
-    </row>
-    <row r="20" ht="13.9" customHeight="1">
-      <c r="B20" s="128" t="inlineStr">
+      <c r="G20" s="91" t="n"/>
+      <c r="I20" s="14" t="n"/>
+    </row>
+    <row r="21" ht="31.5" customHeight="1" s="117">
+      <c r="B21" s="92" t="n"/>
+      <c r="G21" s="91" t="n"/>
+      <c r="I21" s="14" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="88" t="inlineStr">
         <is>
           <t>Escopo: A CAEXPERTS desenvolverá o estudo em 4 etapas, descritas a seguir:
 Na Etapa 1 (Configuração Inicial — 5 dias): Ajuste da geometria 3D da rosca com os parâmetros reais fornecidos pela Braskem (D_screw, D_shaft, pitch, RPM); configuração do domínio DEM no Star-CCM+ 2506 com física de contato Hertz-Mindlin e Liquid Bridge Force (Lian, 1993) para modelar a coesão hexano-PEAD; calibração dos parâmetros de partícula com base na granulometria do PEAD fornecida.
@@ -1899,118 +1828,159 @@
 Na Etapa 4 (Reunião Final Online — dia 25): Apresentação dos resultados e recomendações de mitigação do embuchamento à equipe técnica da Braskem PE5.</t>
         </is>
       </c>
-      <c r="G20" s="124" t="n"/>
-      <c r="I20" s="14" t="n"/>
-    </row>
-    <row r="21" ht="13.9" customHeight="1">
-      <c r="B21" s="128" t="inlineStr">
+      <c r="G22" s="91" t="n"/>
+      <c r="I22" s="14" t="n"/>
+    </row>
+    <row r="23" ht="12.75" customHeight="1" s="117">
+      <c r="B23" s="92" t="n"/>
+      <c r="G23" s="91" t="n"/>
+      <c r="I23" s="14" t="n"/>
+    </row>
+    <row r="24" ht="12.75" customHeight="1" s="117">
+      <c r="B24" s="88" t="inlineStr">
         <is>
           <t>Cronograma de Atividades: A execução do projeto está prevista para ser realizada em 25 dias, conforme cronograma de atividades em anexo. A primeira etapa se iniciará oficialmente a partir do dia subsequente ao recebimento dos documentos com os dados necessários ao projeto. Cada etapa está com a duração em dias prevista conforme indicado abaixo:
 Etapa 1: 5 dias;   Etapa 2: 15 dias;   Etapa 3: 5 dias;   Reunião Final: dia 25.</t>
         </is>
       </c>
-      <c r="G21" s="124" t="n"/>
-      <c r="I21" s="14" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="128" t="inlineStr">
+      <c r="G24" s="91" t="n"/>
+      <c r="I24" s="14" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="92" t="n"/>
+      <c r="G25" s="91" t="n"/>
+      <c r="I25" s="14" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="88" t="inlineStr">
         <is>
           <t>Requisitos/Dados Necessários ao Projeto: Diâmetro externo da pá (D_screw, mm), diâmetro do eixo (D_shaft, mm), passo da hélice (pitch, mm) e RPM de operação; granulometria do pó de PEAD (D10, D50, D90) — alternativamente, confirmação de semelhança com pó de talco; densidade aparente do PEAD (bulk density, kg/m³); localização típica do embuchamento (início/meio/fim da rosca); tipo de rosca em operação (padrão ou cut-flight); e, se disponível, desenho técnico ou croqui com cotas e fotos do equipamento.</t>
         </is>
       </c>
-      <c r="G22" s="124" t="n"/>
-      <c r="I22" s="14" t="n"/>
-    </row>
-    <row r="23" ht="12.75" customHeight="1">
-      <c r="B23" s="128" t="inlineStr">
+      <c r="G26" s="91" t="n"/>
+      <c r="I26" s="14" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="92" t="n"/>
+      <c r="G27" s="91" t="n"/>
+      <c r="I27" s="14" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="88" t="inlineStr">
         <is>
           <t>Entregáveis do Projeto: Relatório técnico em formato .ppt contendo: geometria 3D da rosca simulada (arquivo STEP), campos de velocidade e distribuição de partículas DEM, identificação das zonas de embuchamento, comparação quantitativa entre rosca padrão e cut-flight, e recomendações de mitigação fundamentadas nos resultados das simulações.</t>
         </is>
       </c>
-      <c r="G23" s="124" t="n"/>
-      <c r="I23" s="14" t="n"/>
-    </row>
-    <row r="24" ht="12.75" customHeight="1">
-      <c r="B24" s="128" t="inlineStr">
-        <is>
-          <t>Quem Somos: A CAEXPERTS é uma empresa especializada em digitalização da engenharia que conta com uma rede de consultores pioneiros da implantação de tecnologias de simulação computacional na indústria nacional. Somos parceiros tecnológicos da SIEMENS Digital Industries Software, onde contamos com um portifólio de ferramentas de CAE mais completo do mercado.</t>
-        </is>
-      </c>
-      <c r="G24" s="124" t="n"/>
-      <c r="I24" s="14" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="91" t="inlineStr">
-        <is>
-          <t>INVESTIMENTO TOTAL</t>
-        </is>
-      </c>
-      <c r="C25" s="131" t="n"/>
-      <c r="D25" s="131" t="n"/>
-      <c r="E25" s="131" t="n"/>
-      <c r="F25" s="132">
-        <f>G17</f>
-        <v/>
-      </c>
-      <c r="G25" s="133" t="n"/>
-      <c r="I25" s="14" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="34" t="inlineStr">
-        <is>
-          <t>Observações:</t>
-        </is>
-      </c>
-      <c r="C26" s="15" t="n"/>
-      <c r="D26" s="16" t="n"/>
-      <c r="I26" s="14" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="96" t="inlineStr">
-        <is>
-          <t>Condições de Pagamento: 30 dias.</t>
-        </is>
-      </c>
-      <c r="I27" s="14" t="n"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="96" t="inlineStr">
-        <is>
-          <t>Faturamento: Nota fiscal de serviços</t>
-        </is>
-      </c>
+      <c r="G28" s="91" t="n"/>
       <c r="I28" s="14" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="135" t="inlineStr">
-        <is>
-          <t>Aceitação desta proposta via emissão de pedido de compras ou contrato específico</t>
-        </is>
-      </c>
-      <c r="C29" s="136" t="n"/>
-      <c r="D29" s="136" t="n"/>
-      <c r="E29" s="136" t="n"/>
-      <c r="F29" s="136" t="n"/>
-      <c r="G29" s="137" t="n"/>
+      <c r="B29" s="34" t="n"/>
+      <c r="C29" s="79" t="n"/>
+      <c r="D29" s="7" t="n"/>
+      <c r="E29" s="7" t="n"/>
+      <c r="F29" s="37" t="n"/>
+      <c r="G29" s="36" t="n"/>
+      <c r="I29" s="14" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="88" t="inlineStr">
         <is>
+          <t>Quem Somos: A CAEXPERTS é uma empresa especializada em digitalização da engenharia que conta com uma rede de consultores pioneiros da implantação de tecnologias de simulação computacional na indústria nacional. Somos parceiros tecnológicos da SIEMENS Digital Industries Software, onde contamos com um portifólio de ferramentas de CAE mais completo do mercado.</t>
+        </is>
+      </c>
+      <c r="G30" s="91" t="n"/>
+      <c r="I30" s="14" t="n"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="92" t="n"/>
+      <c r="G31" s="91" t="n"/>
+      <c r="I31" s="14" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="103" t="inlineStr">
+        <is>
+          <t>INVESTIMENTO TOTAL</t>
+        </is>
+      </c>
+      <c r="C32" s="104" t="n"/>
+      <c r="D32" s="104" t="n"/>
+      <c r="E32" s="104" t="n"/>
+      <c r="F32" s="105">
+        <f>G17</f>
+        <v/>
+      </c>
+      <c r="G32" s="106" t="n"/>
+      <c r="I32" s="14" t="n"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="83" t="n"/>
+      <c r="C33" s="26" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="27" t="n"/>
+      <c r="F33" s="27" t="n"/>
+      <c r="G33" s="28" t="n"/>
+      <c r="I33" s="14" t="n"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="33" t="inlineStr">
+        <is>
+          <t>Observações:</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="16" t="n"/>
+      <c r="I34" s="14" t="n"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="95" t="inlineStr">
+        <is>
+          <t>Condições de Pagamento: 30 dias.</t>
+        </is>
+      </c>
+      <c r="I35" s="14" t="n"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="95" t="inlineStr">
+        <is>
+          <t>Faturamento: Nota fiscal de serviços</t>
+        </is>
+      </c>
+      <c r="I36" s="14" t="n"/>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="B38" s="100" t="inlineStr">
+        <is>
+          <t>Aceitação desta proposta via emissão de pedido de compras ou contrato específico</t>
+        </is>
+      </c>
+      <c r="C38" s="101" t="n"/>
+      <c r="D38" s="101" t="n"/>
+      <c r="E38" s="101" t="n"/>
+      <c r="F38" s="101" t="n"/>
+      <c r="G38" s="102" t="n"/>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="B40" s="97" t="inlineStr">
+        <is>
           <t>ANEXO - CRONOGRAMA DE ATIVIDADES</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="12.75" customHeight="1"/>
-    <row r="44" ht="12.75" customHeight="1"/>
-    <row r="45" ht="12.75" customHeight="1"/>
-    <row r="46" ht="12.75" customHeight="1"/>
-    <row r="49" ht="13.9" customHeight="1"/>
-    <row r="52" ht="13.9" customHeight="1"/>
-    <row r="54" ht="13.9" customHeight="1"/>
-    <row r="55" ht="13.9" customHeight="1"/>
-    <row r="56" ht="12.75" customHeight="1"/>
-    <row r="58" ht="15.75" customHeight="1"/>
-    <row r="73" ht="23.25" customHeight="1"/>
+    <row r="43" ht="12.75" customHeight="1" s="117"/>
+    <row r="44" ht="12.75" customHeight="1" s="117"/>
+    <row r="45" ht="12.75" customHeight="1" s="117"/>
+    <row r="46" ht="12.75" customHeight="1" s="117"/>
+    <row r="49" ht="13.9" customHeight="1" s="117"/>
+    <row r="50" ht="34.5" customHeight="1" s="117"/>
+    <row r="52" ht="39.75" customHeight="1" s="117"/>
+    <row r="54" ht="13.9" customHeight="1" s="117"/>
+    <row r="55" ht="13.9" customHeight="1" s="117"/>
+    <row r="56" ht="12.75" customHeight="1" s="117"/>
+    <row r="58" ht="15.75" customHeight="1" s="117"/>
+    <row r="73" ht="23.25" customHeight="1" s="117"/>
   </sheetData>
   <mergeCells count="29">
     <mergeCell ref="E10:G10"/>
@@ -2029,8 +1999,8 @@
     <mergeCell ref="E11:G11"/>
     <mergeCell ref="F15:G15"/>
     <mergeCell ref="F17:F18"/>
+    <mergeCell ref="E7:G7"/>
     <mergeCell ref="B64:G64"/>
-    <mergeCell ref="E7:G7"/>
     <mergeCell ref="B58:E58"/>
     <mergeCell ref="B54:G56"/>
     <mergeCell ref="B23:G24"/>
@@ -2059,500 +2029,619 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:R30"/>
+  <dimension ref="B2:R33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
-    <col width="63.28515625" customWidth="1" min="2" max="2"/>
-    <col width="5.140625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="7" bestFit="1" customWidth="1" min="4" max="7"/>
-    <col width="11.28515625" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="11.28515625" customWidth="1" min="9" max="9"/>
-    <col width="12.140625" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="13.28515625" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="13.28515625" customWidth="1" min="12" max="13"/>
-    <col width="16.5703125" customWidth="1" min="14" max="14"/>
-    <col width="14.7109375" customWidth="1" min="15" max="15"/>
-    <col width="10.7109375" customWidth="1" min="16" max="17"/>
-    <col hidden="1" width="12.28515625" customWidth="1" min="18" max="18"/>
+    <col width="63.28515625" customWidth="1" style="117" min="2" max="2"/>
+    <col width="5.140625" bestFit="1" customWidth="1" style="117" min="3" max="3"/>
+    <col width="7" bestFit="1" customWidth="1" style="117" min="4" max="4"/>
+    <col width="8.7109375" customWidth="1" style="117" min="5" max="5"/>
+    <col width="7" bestFit="1" customWidth="1" style="117" min="6" max="6"/>
+    <col width="8.28515625" customWidth="1" style="117" min="7" max="7"/>
+    <col width="11.28515625" bestFit="1" customWidth="1" style="117" min="8" max="8"/>
+    <col width="11.28515625" customWidth="1" style="117" min="9" max="9"/>
+    <col width="12.140625" bestFit="1" customWidth="1" style="117" min="10" max="10"/>
+    <col width="13.28515625" bestFit="1" customWidth="1" style="117" min="11" max="11"/>
+    <col width="13.28515625" customWidth="1" style="117" min="12" max="13"/>
+    <col width="16.5703125" customWidth="1" style="117" min="14" max="14"/>
+    <col width="14.7109375" customWidth="1" style="117" min="15" max="15"/>
+    <col width="10.7109375" customWidth="1" style="117" min="16" max="17"/>
+    <col hidden="1" width="12.28515625" customWidth="1" style="117" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="2" ht="13.5" customHeight="1" thickBot="1">
-      <c r="N2" s="46" t="n"/>
-      <c r="R2" s="45" t="inlineStr">
+    <row r="2" ht="13.5" customHeight="1" s="117" thickBot="1">
+      <c r="N2" s="45" t="n"/>
+      <c r="R2" s="44" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B3" s="57" t="inlineStr">
+    <row r="3" ht="15.75" customHeight="1" s="117" thickBot="1">
+      <c r="B3" s="56" t="inlineStr">
         <is>
           <t>ATIVIDADES DO PROJETO:                   |                  ETAPAS:</t>
         </is>
       </c>
-      <c r="C3" s="58" t="n">
+      <c r="C3" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="D3" s="59" t="n">
+      <c r="D3" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="59" t="n">
+      <c r="E3" s="58" t="n">
         <v>2</v>
       </c>
-      <c r="F3" s="59" t="n">
+      <c r="F3" s="58" t="n">
         <v>3</v>
       </c>
-      <c r="G3" s="60" t="n">
+      <c r="G3" s="59" t="n">
         <v>4</v>
       </c>
-      <c r="K3" s="46" t="inlineStr">
+      <c r="K3" s="45" t="inlineStr">
         <is>
           <t>Marcus</t>
         </is>
       </c>
-      <c r="L3" s="46" t="inlineStr">
+      <c r="L3" s="45" t="inlineStr">
         <is>
           <t>Gabriel</t>
         </is>
       </c>
-      <c r="M3" s="45" t="n"/>
-      <c r="N3" s="46" t="inlineStr">
+      <c r="M3" s="44" t="n"/>
+      <c r="N3" s="45" t="inlineStr">
         <is>
           <t>Urgência</t>
         </is>
       </c>
-      <c r="O3" s="45" t="inlineStr">
+      <c r="O3" s="44" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="P3" s="50" t="n"/>
-      <c r="Q3" s="50" t="n"/>
-      <c r="R3" s="79" t="inlineStr">
+      <c r="P3" s="49" t="n"/>
+      <c r="Q3" s="49" t="n"/>
+      <c r="R3" s="77" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" thickBot="1" thickTop="1">
-      <c r="B4" s="69" t="inlineStr">
+    <row r="4" ht="16.5" customHeight="1" s="117" thickBot="1" thickTop="1">
+      <c r="B4" s="67" t="inlineStr">
         <is>
           <t>Início de Projeto</t>
         </is>
       </c>
-      <c r="C4" s="70" t="inlineStr">
+      <c r="C4" s="68" t="inlineStr">
         <is>
           <t>dia 0</t>
         </is>
       </c>
-      <c r="D4" s="53" t="n"/>
-      <c r="E4" s="53" t="n"/>
-      <c r="F4" s="53" t="n"/>
-      <c r="G4" s="54" t="n"/>
-      <c r="N4" s="46" t="inlineStr">
+      <c r="D4" s="52" t="n"/>
+      <c r="E4" s="52" t="n"/>
+      <c r="F4" s="52" t="n"/>
+      <c r="G4" s="53" t="n"/>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N4" s="45" t="inlineStr">
         <is>
           <t>Total Eq. Téc.</t>
         </is>
       </c>
-      <c r="O4" s="138">
-        <f>SUM(K24:L24)</f>
-        <v/>
-      </c>
-      <c r="P4" s="50" t="n"/>
-      <c r="Q4" s="50" t="n"/>
-      <c r="R4" s="50" t="n"/>
-    </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="B5" s="63" t="n"/>
-      <c r="C5" s="72" t="n"/>
-      <c r="D5" s="61" t="n"/>
-      <c r="E5" s="73" t="n"/>
-      <c r="F5" s="73" t="n"/>
-      <c r="G5" s="56" t="n"/>
-      <c r="N5" s="46" t="inlineStr">
+      <c r="O4" s="51">
+        <f>SUM(K27:L27)</f>
+        <v/>
+      </c>
+      <c r="P4" s="49" t="n"/>
+      <c r="Q4" s="49" t="n"/>
+      <c r="R4" s="49" t="n"/>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="117">
+      <c r="B5" s="62" t="inlineStr">
+        <is>
+          <t>Recebimento das informações e documentos do projeto</t>
+        </is>
+      </c>
+      <c r="C5" s="70" t="n"/>
+      <c r="D5" s="60" t="n"/>
+      <c r="E5" s="71" t="n"/>
+      <c r="F5" s="71" t="n"/>
+      <c r="G5" s="55" t="n"/>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>8</v>
+      </c>
+      <c r="N5" s="45" t="inlineStr">
         <is>
           <t>Total Projeto:</t>
         </is>
       </c>
-      <c r="O5" s="138">
+      <c r="O5" s="51">
         <f>O4/0.35</f>
         <v/>
       </c>
-      <c r="P5" s="139" t="n"/>
-      <c r="Q5" s="139" t="n"/>
-      <c r="R5" s="140" t="inlineStr">
+      <c r="P5" s="50" t="n"/>
+      <c r="Q5" s="50" t="n"/>
+      <c r="R5" s="78" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="B6" s="55" t="n"/>
-      <c r="C6" s="72" t="n"/>
-      <c r="D6" s="62" t="n"/>
-      <c r="E6" s="73" t="n"/>
-      <c r="F6" s="73" t="n"/>
-      <c r="G6" s="56" t="n"/>
-      <c r="N6" s="50" t="inlineStr">
+    <row r="6" ht="15" customHeight="1" s="117">
+      <c r="B6" s="54" t="inlineStr">
+        <is>
+          <t>Revisão da literatura normas aplicáveis e documentos do projeto</t>
+        </is>
+      </c>
+      <c r="C6" s="70" t="n"/>
+      <c r="D6" s="61" t="n"/>
+      <c r="E6" s="71" t="n"/>
+      <c r="F6" s="71" t="n"/>
+      <c r="G6" s="55" t="n"/>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" s="49" t="inlineStr">
         <is>
           <t>Rateio</t>
         </is>
       </c>
-      <c r="O6" s="84" t="n">
+      <c r="O6" s="82" t="n">
         <v>0.35</v>
       </c>
-      <c r="P6" s="139" t="n"/>
-      <c r="Q6" s="139" t="n"/>
-      <c r="R6" s="140" t="inlineStr">
+      <c r="P6" s="50" t="n"/>
+      <c r="Q6" s="50" t="n"/>
+      <c r="R6" s="78" t="inlineStr">
         <is>
           <t>CFD + DEM</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="B7" s="55" t="n"/>
-      <c r="C7" s="72" t="n"/>
-      <c r="D7" s="62" t="n"/>
-      <c r="E7" s="73" t="n"/>
-      <c r="F7" s="73" t="n"/>
-      <c r="G7" s="56" t="n"/>
-      <c r="N7" s="50" t="n"/>
-      <c r="O7" s="139" t="n"/>
-      <c r="P7" s="139" t="n"/>
-      <c r="Q7" s="139" t="n"/>
-      <c r="R7" s="140" t="inlineStr">
+    <row r="7" ht="15" customHeight="1" s="117">
+      <c r="B7" s="54" t="inlineStr">
+        <is>
+          <t>Simplificação do CAD 3D para simulação CFD</t>
+        </is>
+      </c>
+      <c r="C7" s="70" t="n"/>
+      <c r="D7" s="61" t="n"/>
+      <c r="E7" s="71" t="n"/>
+      <c r="F7" s="71" t="n"/>
+      <c r="G7" s="55" t="n"/>
+      <c r="K7" t="n">
+        <v>2</v>
+      </c>
+      <c r="L7" t="n">
+        <v>4</v>
+      </c>
+      <c r="N7" s="49" t="n"/>
+      <c r="O7" s="50" t="n"/>
+      <c r="P7" s="50" t="n"/>
+      <c r="Q7" s="50" t="n"/>
+      <c r="R7" s="78" t="inlineStr">
         <is>
           <t>FEA</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B8" s="55" t="n"/>
-      <c r="C8" s="72" t="n"/>
-      <c r="D8" s="62" t="n"/>
-      <c r="E8" s="73" t="n"/>
-      <c r="F8" s="73" t="n"/>
-      <c r="G8" s="56" t="n"/>
-      <c r="N8" s="50" t="n"/>
-      <c r="O8" s="139" t="n"/>
-      <c r="P8" s="139" t="n"/>
-      <c r="Q8" s="139" t="n"/>
-      <c r="R8" s="140" t="inlineStr">
+    <row r="8" ht="15" customHeight="1" s="117">
+      <c r="B8" s="54" t="inlineStr">
+        <is>
+          <t>Definição das premissas e dos cenários de análise</t>
+        </is>
+      </c>
+      <c r="C8" s="70" t="n"/>
+      <c r="D8" s="61" t="n"/>
+      <c r="E8" s="71" t="n"/>
+      <c r="F8" s="71" t="n"/>
+      <c r="G8" s="55" t="n"/>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" s="49" t="n"/>
+      <c r="O8" s="50" t="n"/>
+      <c r="P8" s="50" t="n"/>
+      <c r="Q8" s="50" t="n"/>
+      <c r="R8" s="78" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="117">
+      <c r="B9" s="54" t="inlineStr">
+        <is>
+          <t>Criação da planilha de projeto</t>
+        </is>
+      </c>
+      <c r="C9" s="70" t="n"/>
+      <c r="D9" s="61" t="n"/>
+      <c r="E9" s="71" t="n"/>
+      <c r="F9" s="71" t="n"/>
+      <c r="G9" s="55" t="n"/>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" s="49" t="n"/>
+      <c r="O9" s="50" t="n"/>
+      <c r="P9" s="50" t="n"/>
+      <c r="Q9" s="50" t="n"/>
+      <c r="R9" s="78" t="n"/>
+    </row>
+    <row r="10" ht="15.75" customHeight="1" s="117" thickBot="1">
+      <c r="B10" s="54" t="inlineStr">
+        <is>
+          <t>Kick-off Meeting</t>
+        </is>
+      </c>
+      <c r="C10" s="70" t="n"/>
+      <c r="D10" s="61" t="n"/>
+      <c r="E10" s="71" t="n"/>
+      <c r="F10" s="71" t="n"/>
+      <c r="G10" s="55" t="n"/>
+      <c r="N10" s="49" t="n"/>
+      <c r="O10" s="50" t="n"/>
+      <c r="P10" s="50" t="n"/>
+      <c r="Q10" s="50" t="n"/>
+      <c r="R10" s="78" t="inlineStr">
         <is>
           <t>EMAG</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B9" s="66" t="inlineStr">
+    <row r="11" ht="15.75" customHeight="1" s="117" thickBot="1">
+      <c r="B11" s="64" t="inlineStr">
         <is>
           <t>Configuração Inicial</t>
         </is>
       </c>
-      <c r="C9" s="67" t="n"/>
-      <c r="D9" s="70">
-        <f>"+" &amp; $H9 &amp; " dias"</f>
-        <v/>
-      </c>
-      <c r="E9" s="73" t="n"/>
-      <c r="F9" s="73" t="n"/>
-      <c r="G9" s="56" t="n"/>
-      <c r="H9" t="n">
+      <c r="C11" s="65" t="n"/>
+      <c r="D11" s="68">
+        <f>"+" &amp; $H11 &amp; " dias"</f>
+        <v/>
+      </c>
+      <c r="E11" s="71" t="n"/>
+      <c r="F11" s="71" t="n"/>
+      <c r="G11" s="55" t="n"/>
+      <c r="H11" t="n">
         <v>5</v>
       </c>
-      <c r="N9" s="141" t="n"/>
-    </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="B10" s="63" t="inlineStr">
+      <c r="N11" s="46" t="n"/>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="117">
+      <c r="B12" s="62" t="inlineStr">
         <is>
           <t>Ajuste da geometria 3D (D_screw, D_shaft, pitch) com parâmetros reais Braskem</t>
         </is>
       </c>
-      <c r="C10" s="65" t="n"/>
-      <c r="D10" s="73" t="n"/>
-      <c r="E10" s="61" t="n"/>
-      <c r="F10" s="73" t="n"/>
-      <c r="G10" s="56" t="n"/>
-      <c r="L10" t="n">
+      <c r="C12" s="63" t="n"/>
+      <c r="D12" s="71" t="n"/>
+      <c r="E12" s="60" t="n"/>
+      <c r="F12" s="71" t="n"/>
+      <c r="G12" s="55" t="n"/>
+      <c r="K12" t="n">
         <v>2</v>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="B11" s="55" t="inlineStr">
-        <is>
-          <t>Setup DEM no Star-CCM+ 2506: Hertz-Mindlin + Liquid Bridge Force (Lian, 1993)</t>
-        </is>
-      </c>
-      <c r="C11" s="73" t="n"/>
-      <c r="D11" s="73" t="n"/>
-      <c r="E11" s="62" t="n"/>
-      <c r="F11" s="73" t="n"/>
-      <c r="G11" s="56" t="n"/>
-      <c r="K11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B12" s="55" t="inlineStr">
-        <is>
-          <t>Calibração dos parâmetros de partícula (granulometria + bulk density do PEAD)</t>
-        </is>
-      </c>
-      <c r="C12" s="73" t="n"/>
-      <c r="D12" s="73" t="n"/>
-      <c r="E12" s="62" t="n"/>
-      <c r="F12" s="73" t="n"/>
-      <c r="G12" s="56" t="n"/>
-      <c r="K12" t="n">
-        <v>1</v>
       </c>
       <c r="L12" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="13" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B13" s="66" t="inlineStr">
+    <row r="13" ht="15" customHeight="1" s="117">
+      <c r="B13" s="54" t="inlineStr">
+        <is>
+          <t>Setup DEM no Star-CCM+</t>
+        </is>
+      </c>
+      <c r="C13" s="71" t="n"/>
+      <c r="D13" s="71" t="n"/>
+      <c r="E13" s="61" t="n"/>
+      <c r="F13" s="71" t="n"/>
+      <c r="G13" s="55" t="n"/>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" ht="15.75" customHeight="1" s="117" thickBot="1">
+      <c r="B14" s="54" t="inlineStr">
+        <is>
+          <t>Calibração dos parâmetros de partícula (granulometria + bulk density do PEAD)</t>
+        </is>
+      </c>
+      <c r="C14" s="71" t="n"/>
+      <c r="D14" s="71" t="n"/>
+      <c r="E14" s="61" t="n"/>
+      <c r="F14" s="71" t="n"/>
+      <c r="G14" s="55" t="n"/>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" ht="15.75" customHeight="1" s="117" thickBot="1">
+      <c r="B15" s="64" t="inlineStr">
         <is>
           <t>Simulações dos Cenários</t>
         </is>
       </c>
-      <c r="C13" s="68" t="n"/>
-      <c r="D13" s="68" t="n"/>
-      <c r="E13" s="70">
-        <f>"+" &amp; $H13 &amp; " dias"</f>
-        <v/>
-      </c>
-      <c r="F13" s="73" t="n"/>
-      <c r="G13" s="56" t="n"/>
-      <c r="H13" t="n">
+      <c r="C15" s="66" t="n"/>
+      <c r="D15" s="66" t="n"/>
+      <c r="E15" s="68">
+        <f>"+" &amp; $H15 &amp; " dias"</f>
+        <v/>
+      </c>
+      <c r="F15" s="71" t="n"/>
+      <c r="G15" s="55" t="n"/>
+      <c r="H15" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="B14" s="63" t="inlineStr">
+    <row r="16" ht="15" customHeight="1" s="117">
+      <c r="B16" s="62" t="inlineStr">
         <is>
           <t>Caso 1 — Rosca padrão: análise de zonas de velocidade ≈ 0 (embuchamento)</t>
         </is>
       </c>
-      <c r="C14" s="73" t="n"/>
-      <c r="D14" s="73" t="n"/>
-      <c r="E14" s="73" t="n"/>
-      <c r="F14" s="61" t="n"/>
-      <c r="G14" s="56" t="n"/>
-      <c r="L14" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="B15" s="55" t="inlineStr">
-        <is>
-          <t>Caso 2 — Rosca cut-flight: comparação com o caso base</t>
-        </is>
-      </c>
-      <c r="C15" s="73" t="n"/>
-      <c r="D15" s="73" t="n"/>
-      <c r="E15" s="73" t="n"/>
-      <c r="F15" s="62" t="n"/>
-      <c r="G15" s="56" t="n"/>
-      <c r="L15" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B16" s="55" t="inlineStr">
-        <is>
-          <t>Análise de campos de pressão e tensão sobre as partículas DEM</t>
-        </is>
-      </c>
-      <c r="C16" s="73" t="n"/>
-      <c r="D16" s="73" t="n"/>
-      <c r="E16" s="73" t="n"/>
-      <c r="F16" s="62" t="n"/>
-      <c r="G16" s="56" t="n"/>
+      <c r="C16" s="71" t="n"/>
+      <c r="D16" s="71" t="n"/>
+      <c r="E16" s="71" t="n"/>
+      <c r="F16" s="60" t="n"/>
+      <c r="G16" s="55" t="n"/>
       <c r="K16" t="n">
         <v>2</v>
       </c>
       <c r="L16" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="117">
+      <c r="B17" s="54" t="inlineStr">
+        <is>
+          <t>Caso 2 — Rosca cut-flight: comparação com o caso base</t>
+        </is>
+      </c>
+      <c r="C17" s="71" t="n"/>
+      <c r="D17" s="71" t="n"/>
+      <c r="E17" s="71" t="n"/>
+      <c r="F17" s="61" t="n"/>
+      <c r="G17" s="55" t="n"/>
+      <c r="K17" t="n">
+        <v>3</v>
+      </c>
+      <c r="L17" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1" s="117" thickBot="1">
+      <c r="B18" s="54" t="inlineStr">
+        <is>
+          <t>Análise de campos de pressão sobre as partículas DEM</t>
+        </is>
+      </c>
+      <c r="C18" s="71" t="n"/>
+      <c r="D18" s="71" t="n"/>
+      <c r="E18" s="71" t="n"/>
+      <c r="F18" s="61" t="n"/>
+      <c r="G18" s="55" t="n"/>
+      <c r="K18" t="n">
+        <v>2</v>
+      </c>
+      <c r="L18" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B17" s="66" t="inlineStr">
+    <row r="19" ht="15.75" customHeight="1" s="117" thickBot="1">
+      <c r="B19" s="64" t="inlineStr">
         <is>
           <t>Finalização</t>
         </is>
       </c>
-      <c r="C17" s="68" t="n"/>
-      <c r="D17" s="68" t="n"/>
-      <c r="E17" s="68" t="n"/>
-      <c r="F17" s="70">
-        <f>"+" &amp; $H17 &amp; " dias"</f>
-        <v/>
-      </c>
-      <c r="G17" s="56" t="n"/>
-      <c r="H17" t="n">
+      <c r="C19" s="66" t="n"/>
+      <c r="D19" s="66" t="n"/>
+      <c r="E19" s="66" t="n"/>
+      <c r="F19" s="68">
+        <f>"+" &amp; $H19 &amp; " dias"</f>
+        <v/>
+      </c>
+      <c r="G19" s="55" t="n"/>
+      <c r="H19" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="B18" s="55" t="inlineStr">
+    <row r="20" ht="15" customHeight="1" s="117">
+      <c r="B20" s="54" t="inlineStr">
         <is>
           <t>Pós-processamento: campos de velocidade, pressão e distribuição de partículas</t>
         </is>
       </c>
-      <c r="C18" s="73" t="n"/>
-      <c r="D18" s="73" t="n"/>
-      <c r="E18" s="73" t="n"/>
-      <c r="F18" s="73" t="n"/>
-      <c r="G18" s="62" t="n"/>
-      <c r="L18" t="n">
+      <c r="C20" s="71" t="n"/>
+      <c r="D20" s="71" t="n"/>
+      <c r="E20" s="71" t="n"/>
+      <c r="F20" s="71" t="n"/>
+      <c r="G20" s="61" t="n"/>
+      <c r="K20" t="n">
+        <v>2</v>
+      </c>
+      <c r="L20" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="B19" s="55" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="117">
+      <c r="B21" s="54" t="inlineStr">
         <is>
           <t>Comparação quantitativa rosca padrão vs. cut-flight + identificação de zonas críticas</t>
         </is>
       </c>
-      <c r="C19" s="73" t="n"/>
-      <c r="D19" s="73" t="n"/>
-      <c r="E19" s="73" t="n"/>
-      <c r="F19" s="73" t="n"/>
-      <c r="G19" s="62" t="n"/>
-      <c r="K19" t="n">
+      <c r="C21" s="71" t="n"/>
+      <c r="D21" s="71" t="n"/>
+      <c r="E21" s="71" t="n"/>
+      <c r="F21" s="71" t="n"/>
+      <c r="G21" s="61" t="n"/>
+      <c r="K21" t="n">
         <v>1</v>
       </c>
-      <c r="L19" t="n">
+      <c r="L21" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B20" s="64" t="inlineStr">
+    <row r="22" ht="15" customHeight="1" s="117">
+      <c r="B22" s="54" t="inlineStr">
         <is>
           <t>Elaboração do relatório técnico em formato .ppt com metodologia e recomendações</t>
         </is>
       </c>
-      <c r="C20" s="73" t="n"/>
-      <c r="D20" s="73" t="n"/>
-      <c r="E20" s="73" t="n"/>
-      <c r="F20" s="73" t="n"/>
-      <c r="G20" s="62" t="n"/>
-      <c r="K20" t="n">
+      <c r="C22" s="71" t="n"/>
+      <c r="D22" s="71" t="n"/>
+      <c r="E22" s="71" t="n"/>
+      <c r="F22" s="71" t="n"/>
+      <c r="G22" s="61" t="n"/>
+      <c r="K22" t="n">
         <v>1</v>
       </c>
-      <c r="L20" t="n">
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="117" thickBot="1">
+      <c r="B23" s="114" t="inlineStr">
+        <is>
+          <t>Kit de Entregas</t>
+        </is>
+      </c>
+      <c r="C23" s="71" t="n"/>
+      <c r="D23" s="71" t="n"/>
+      <c r="E23" s="71" t="n"/>
+      <c r="F23" s="71" t="n"/>
+      <c r="G23" s="61" t="n"/>
+      <c r="K23" t="n">
+        <v>1</v>
+      </c>
+      <c r="L23" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B21" s="66" t="inlineStr">
+    <row r="24" ht="15.75" customHeight="1" s="117" thickBot="1">
+      <c r="B24" s="64" t="inlineStr">
         <is>
           <t>Reunião Final Online</t>
         </is>
       </c>
-      <c r="C21" s="68" t="n"/>
-      <c r="D21" s="68" t="n"/>
-      <c r="E21" s="68" t="n"/>
-      <c r="F21" s="68" t="n"/>
-      <c r="G21" s="70">
-        <f>"+" &amp; $H21 &amp; " dias"</f>
-        <v/>
-      </c>
-      <c r="H21" t="n">
+      <c r="C24" s="66" t="n"/>
+      <c r="D24" s="66" t="n"/>
+      <c r="E24" s="66" t="n"/>
+      <c r="F24" s="66" t="n"/>
+      <c r="G24" s="68">
+        <f>"+" &amp; $H24 &amp; " dias"</f>
+        <v/>
+      </c>
+      <c r="H24" t="n">
         <v>25</v>
       </c>
-      <c r="K21" t="n">
+      <c r="K24" t="n">
         <v>2</v>
       </c>
-      <c r="L21" t="n">
+      <c r="L24" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="22">
-      <c r="H22">
-        <f>SUM(H5:H21)</f>
-        <v/>
-      </c>
-      <c r="J22" s="46" t="inlineStr">
+    <row r="25">
+      <c r="H25">
+        <f>SUM(H5:H24)</f>
+        <v/>
+      </c>
+      <c r="J25" s="45" t="inlineStr">
         <is>
           <t>Total Horas</t>
         </is>
       </c>
-      <c r="K22">
-        <f>SUM(K4:K21)</f>
-        <v/>
-      </c>
-      <c r="L22">
-        <f>SUM(L4:L21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="J23" s="46" t="inlineStr">
+      <c r="K25">
+        <f>SUM(K4:K24)</f>
+        <v/>
+      </c>
+      <c r="L25">
+        <f>SUM(L4:L24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="J26" s="45" t="inlineStr">
         <is>
           <t>Valor HH</t>
         </is>
       </c>
-      <c r="K23" s="141">
+      <c r="K26" s="46">
         <f>VLOOKUP(K3,'Tabela HH'!$H$4:$K$19,IF($O$3="Sim",4,3),0)</f>
         <v/>
       </c>
-      <c r="L23" s="141">
+      <c r="L26" s="46">
         <f>VLOOKUP(L3,'Tabela HH'!$H$4:$K$19,IF($O$3="Sim",4,3),0)</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="K24" s="138">
-        <f>K22*VLOOKUP(K3,'Tabela HH'!$H$4:$K$19,IF($O$3="Sim",4,3),0)</f>
-        <v/>
-      </c>
-      <c r="L24" s="138">
-        <f>L22*VLOOKUP(L3,'Tabela HH'!$H$4:$K$19,IF($O$3="Sim",4,3),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="J25" s="46" t="inlineStr">
+    <row r="27">
+      <c r="K27" s="51">
+        <f>K25*VLOOKUP(K3,'Tabela HH'!$H$4:$K$19,IF($O$3="Sim",4,3),0)</f>
+        <v/>
+      </c>
+      <c r="L27" s="51">
+        <f>L25*VLOOKUP(L3,'Tabela HH'!$H$4:$K$19,IF($O$3="Sim",4,3),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="J28" s="45" t="inlineStr">
         <is>
           <t>% Calculado</t>
         </is>
       </c>
-      <c r="K25" s="142">
-        <f>K24/$O$4*$O$6</f>
-        <v/>
-      </c>
-      <c r="L25" s="142">
-        <f>L24/$O$4*$O$6</f>
-        <v/>
-      </c>
-      <c r="M25" s="74">
-        <f>SUM(K25:L25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="C26" s="45" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="45" t="n"/>
-      <c r="C27" s="45" t="n"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="45" t="n"/>
+      <c r="K28" s="73">
+        <f>K27/$O$4*$O$6</f>
+        <v/>
+      </c>
+      <c r="L28" s="73">
+        <f>L27/$O$4*$O$6</f>
+        <v/>
+      </c>
+      <c r="M28" s="72">
+        <f>SUM(K28:L28)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
-      <c r="B29" s="45" t="n"/>
-    </row>
-    <row r="30" ht="15" customHeight="1">
-      <c r="B30" s="48" t="n"/>
+      <c r="C29" s="44" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="44" t="n"/>
+      <c r="C30" s="44" t="n"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="44" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="44" t="n"/>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="117">
+      <c r="B33" s="47" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation sqref="O3" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>SimNao</formula1>
     </dataValidation>
@@ -2571,611 +2660,611 @@
   <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
-    <col width="16.140625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="13.28515625" customWidth="1" min="3" max="3"/>
-    <col width="12.85546875" customWidth="1" min="4" max="4"/>
-    <col width="10.5703125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="9.85546875" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="12.140625" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="10.7109375" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="11.28515625" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="16.140625" bestFit="1" customWidth="1" style="117" min="1" max="1"/>
+    <col width="12" customWidth="1" style="117" min="2" max="2"/>
+    <col width="13.28515625" customWidth="1" style="117" min="3" max="3"/>
+    <col width="12.85546875" customWidth="1" style="117" min="4" max="4"/>
+    <col width="10.5703125" bestFit="1" customWidth="1" style="117" min="5" max="5"/>
+    <col width="9.85546875" bestFit="1" customWidth="1" style="117" min="8" max="8"/>
+    <col width="12.140625" bestFit="1" customWidth="1" style="117" min="9" max="9"/>
+    <col width="10.7109375" bestFit="1" customWidth="1" style="117" min="10" max="10"/>
+    <col width="11.28515625" bestFit="1" customWidth="1" style="117" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="114" t="inlineStr">
+      <c r="A1" s="111" t="inlineStr">
         <is>
           <t>HH Projetos Geral; Acima de 60 dias de duração e HH de Viagens</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="49" t="n"/>
-      <c r="B2" s="50" t="inlineStr">
+      <c r="A2" s="48" t="n"/>
+      <c r="B2" s="49" t="inlineStr">
         <is>
           <t>CAD</t>
         </is>
       </c>
-      <c r="C2" s="50" t="inlineStr">
+      <c r="C2" s="49" t="inlineStr">
         <is>
           <t>FEA</t>
         </is>
       </c>
-      <c r="D2" s="50" t="inlineStr">
+      <c r="D2" s="49" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
-      <c r="E2" s="50" t="inlineStr">
+      <c r="E2" s="49" t="inlineStr">
         <is>
           <t>EMAG</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="50" t="inlineStr">
+      <c r="A3" s="49" t="inlineStr">
         <is>
           <t>Estagiário</t>
         </is>
       </c>
-      <c r="B3" s="139" t="n">
+      <c r="B3" s="50" t="n">
         <v>15</v>
       </c>
-      <c r="C3" s="139" t="n">
+      <c r="C3" s="50" t="n">
         <v>20</v>
       </c>
-      <c r="D3" s="139" t="n">
+      <c r="D3" s="50" t="n">
         <v>30</v>
       </c>
-      <c r="E3" s="139" t="n">
+      <c r="E3" s="50" t="n">
         <v>30</v>
       </c>
-      <c r="H3" s="46" t="inlineStr">
+      <c r="H3" s="45" t="inlineStr">
         <is>
           <t>Equipe</t>
         </is>
       </c>
-      <c r="I3" s="46" t="inlineStr">
+      <c r="I3" s="45" t="inlineStr">
         <is>
           <t>Senioridade</t>
         </is>
       </c>
-      <c r="J3" s="46" t="inlineStr">
+      <c r="J3" s="45" t="inlineStr">
         <is>
           <t>HH Normal</t>
         </is>
       </c>
-      <c r="K3" s="46" t="inlineStr">
+      <c r="K3" s="45" t="inlineStr">
         <is>
           <t>HH Urgente</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="50" t="inlineStr">
+      <c r="A4" s="49" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="B4" s="139" t="n">
+      <c r="B4" s="50" t="n">
         <v>30</v>
       </c>
-      <c r="C4" s="139" t="n">
+      <c r="C4" s="50" t="n">
         <v>40</v>
       </c>
-      <c r="D4" s="139" t="n">
+      <c r="D4" s="50" t="n">
         <v>50</v>
       </c>
-      <c r="E4" s="139" t="n">
+      <c r="E4" s="50" t="n">
         <v>50</v>
       </c>
-      <c r="G4" s="50" t="n"/>
-      <c r="H4" s="45" t="inlineStr">
+      <c r="G4" s="49" t="n"/>
+      <c r="H4" s="44" t="inlineStr">
         <is>
           <t>Marcus</t>
         </is>
       </c>
-      <c r="I4" s="45" t="inlineStr">
+      <c r="I4" s="44" t="inlineStr">
         <is>
           <t>Senior</t>
         </is>
       </c>
-      <c r="J4" s="141">
+      <c r="J4" s="46">
         <f>VLOOKUP(I4,$A$3:$E$6,4,0)</f>
         <v/>
       </c>
-      <c r="K4" s="141">
+      <c r="K4" s="46">
         <f>VLOOKUP(I4,$A$12:$E$15,4,0)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="50" t="inlineStr">
+      <c r="A5" s="49" t="inlineStr">
         <is>
           <t>Pleno</t>
         </is>
       </c>
-      <c r="B5" s="139" t="n">
+      <c r="B5" s="50" t="n">
         <v>50</v>
       </c>
-      <c r="C5" s="139" t="n">
+      <c r="C5" s="50" t="n">
         <v>60</v>
       </c>
-      <c r="D5" s="139">
+      <c r="D5" s="50">
         <f>75</f>
         <v/>
       </c>
-      <c r="E5" s="139" t="n">
+      <c r="E5" s="50" t="n">
         <v>75</v>
       </c>
-      <c r="G5" s="50" t="n"/>
-      <c r="H5" s="79" t="inlineStr">
+      <c r="G5" s="49" t="n"/>
+      <c r="H5" s="77" t="inlineStr">
         <is>
           <t>Matheus</t>
         </is>
       </c>
-      <c r="I5" s="45" t="inlineStr">
+      <c r="I5" s="44" t="inlineStr">
         <is>
           <t>Pleno</t>
         </is>
       </c>
-      <c r="J5" s="141">
+      <c r="J5" s="46">
         <f>VLOOKUP(I5,$A$3:$E$6,4,0)</f>
         <v/>
       </c>
-      <c r="K5" s="141">
+      <c r="K5" s="46">
         <f>VLOOKUP(I5,$A$12:$E$15,4,0)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="50" t="inlineStr">
+      <c r="A6" s="49" t="inlineStr">
         <is>
           <t>Senior</t>
         </is>
       </c>
-      <c r="B6" s="139" t="n">
+      <c r="B6" s="50" t="n">
         <v>80</v>
       </c>
-      <c r="C6" s="139">
+      <c r="C6" s="50">
         <f>90</f>
         <v/>
       </c>
-      <c r="D6" s="139">
+      <c r="D6" s="50">
         <f>100</f>
         <v/>
       </c>
-      <c r="E6" s="139" t="n">
+      <c r="E6" s="50" t="n">
         <v>100</v>
       </c>
-      <c r="G6" s="50" t="n"/>
-      <c r="H6" s="45" t="inlineStr">
+      <c r="G6" s="49" t="n"/>
+      <c r="H6" s="44" t="inlineStr">
         <is>
           <t>Otávio</t>
         </is>
       </c>
-      <c r="I6" s="45" t="inlineStr">
+      <c r="I6" s="44" t="inlineStr">
         <is>
           <t>Pleno</t>
         </is>
       </c>
-      <c r="J6" s="141">
+      <c r="J6" s="46">
         <f>VLOOKUP(I6,$A$3:$E$6,4,0)</f>
         <v/>
       </c>
-      <c r="K6" s="141">
+      <c r="K6" s="46">
         <f>VLOOKUP(I6,$A$12:$E$15,4,0)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="G7" s="50" t="n"/>
-      <c r="H7" s="45" t="inlineStr">
+      <c r="G7" s="49" t="n"/>
+      <c r="H7" s="44" t="inlineStr">
         <is>
           <t>Humberto</t>
         </is>
       </c>
-      <c r="I7" s="45" t="inlineStr">
+      <c r="I7" s="44" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="J7" s="141">
+      <c r="J7" s="46">
         <f>VLOOKUP(I7,$A$3:$E$6,4,0)</f>
         <v/>
       </c>
-      <c r="K7" s="141">
+      <c r="K7" s="46">
         <f>VLOOKUP(I7,$A$12:$E$15,4,0)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="G8" s="50" t="n"/>
-      <c r="H8" s="45" t="inlineStr">
+      <c r="G8" s="49" t="n"/>
+      <c r="H8" s="44" t="inlineStr">
         <is>
           <t>João</t>
         </is>
       </c>
-      <c r="I8" s="45" t="inlineStr">
+      <c r="I8" s="44" t="inlineStr">
         <is>
           <t>Estagiário</t>
         </is>
       </c>
-      <c r="J8" s="141">
+      <c r="J8" s="46">
         <f>VLOOKUP(I8,$A$3:$E$6,4,0)</f>
         <v/>
       </c>
-      <c r="K8" s="141">
+      <c r="K8" s="46">
         <f>VLOOKUP(I8,$A$12:$E$15,4,0)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="114" t="inlineStr">
+      <c r="A9" s="111" t="inlineStr">
         <is>
           <t>HH Projetos Geral; Abaixo de 60 dias de duração ou urgentes</t>
         </is>
       </c>
-      <c r="G9" s="50" t="n"/>
-      <c r="H9" s="45" t="inlineStr">
+      <c r="G9" s="49" t="n"/>
+      <c r="H9" s="44" t="inlineStr">
         <is>
           <t>Vitor</t>
         </is>
       </c>
-      <c r="I9" s="45" t="inlineStr">
+      <c r="I9" s="44" t="inlineStr">
         <is>
           <t>Estagiário</t>
         </is>
       </c>
-      <c r="J9" s="141">
+      <c r="J9" s="46">
         <f>VLOOKUP(I9,$A$3:$E$6,4,0)</f>
         <v/>
       </c>
-      <c r="K9" s="141">
+      <c r="K9" s="46">
         <f>VLOOKUP(I9,$A$12:$E$15,4,0)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="114" t="n"/>
-      <c r="B10" s="114" t="n"/>
-      <c r="C10" s="114" t="n"/>
-      <c r="D10" s="114" t="n"/>
-      <c r="E10" s="114" t="n"/>
-      <c r="G10" s="50" t="n"/>
-      <c r="H10" s="45" t="inlineStr">
+      <c r="A10" s="111" t="n"/>
+      <c r="B10" s="111" t="n"/>
+      <c r="C10" s="111" t="n"/>
+      <c r="D10" s="111" t="n"/>
+      <c r="E10" s="111" t="n"/>
+      <c r="G10" s="49" t="n"/>
+      <c r="H10" s="44" t="inlineStr">
         <is>
           <t>Gabriel</t>
         </is>
       </c>
-      <c r="I10" s="45" t="inlineStr">
+      <c r="I10" s="44" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="J10" s="141">
+      <c r="J10" s="46">
         <f>VLOOKUP(I10,$A$3:$E$6,4,0)</f>
         <v/>
       </c>
-      <c r="K10" s="141">
+      <c r="K10" s="46">
         <f>VLOOKUP(I10,$A$12:$E$15,4,0)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="49" t="n"/>
-      <c r="B11" s="50" t="inlineStr">
+      <c r="A11" s="48" t="n"/>
+      <c r="B11" s="49" t="inlineStr">
         <is>
           <t>CAD</t>
         </is>
       </c>
-      <c r="C11" s="50" t="inlineStr">
+      <c r="C11" s="49" t="inlineStr">
         <is>
           <t>FEA</t>
         </is>
       </c>
-      <c r="D11" s="50" t="inlineStr">
+      <c r="D11" s="49" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
-      <c r="E11" s="50" t="inlineStr">
+      <c r="E11" s="49" t="inlineStr">
         <is>
           <t>EMAG</t>
         </is>
       </c>
-      <c r="G11" s="114" t="n"/>
-      <c r="H11" s="79" t="inlineStr">
+      <c r="G11" s="111" t="n"/>
+      <c r="H11" s="77" t="inlineStr">
         <is>
           <t>Vinicius</t>
         </is>
       </c>
-      <c r="I11" s="45" t="inlineStr">
+      <c r="I11" s="44" t="inlineStr">
         <is>
           <t>Estagiário</t>
         </is>
       </c>
-      <c r="J11" s="141">
+      <c r="J11" s="46">
         <f>VLOOKUP(I11,$A$3:$E$6,4,0)</f>
         <v/>
       </c>
-      <c r="K11" s="141">
+      <c r="K11" s="46">
         <f>VLOOKUP(I11,$A$12:$E$15,4,0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="50" t="inlineStr">
+      <c r="A12" s="49" t="inlineStr">
         <is>
           <t>Estagiário</t>
         </is>
       </c>
-      <c r="B12" s="139">
+      <c r="B12" s="50">
         <f>1.4*B3</f>
         <v/>
       </c>
-      <c r="C12" s="139">
+      <c r="C12" s="50">
         <f>1.4*C3</f>
         <v/>
       </c>
-      <c r="D12" s="139">
+      <c r="D12" s="50">
         <f>1.4*D3</f>
         <v/>
       </c>
-      <c r="E12" s="139">
+      <c r="E12" s="50">
         <f>1.4*E3</f>
         <v/>
       </c>
-      <c r="G12" s="50" t="n"/>
-      <c r="H12" s="45" t="inlineStr">
+      <c r="G12" s="49" t="n"/>
+      <c r="H12" s="44" t="inlineStr">
         <is>
           <t>Guerra</t>
         </is>
       </c>
-      <c r="I12" s="45" t="inlineStr">
+      <c r="I12" s="44" t="inlineStr">
         <is>
           <t>Externo</t>
         </is>
       </c>
-      <c r="J12" s="141" t="n">
+      <c r="J12" s="46" t="n">
         <v>120</v>
       </c>
-      <c r="K12" s="141" t="n">
+      <c r="K12" s="46" t="n">
         <v>120</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="50" t="inlineStr">
+      <c r="A13" s="49" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="B13" s="139">
+      <c r="B13" s="50">
         <f>1.4*B4</f>
         <v/>
       </c>
-      <c r="C13" s="139">
+      <c r="C13" s="50">
         <f>1.4*C4</f>
         <v/>
       </c>
-      <c r="D13" s="139">
+      <c r="D13" s="50">
         <f>1.4*D4</f>
         <v/>
       </c>
-      <c r="E13" s="139">
+      <c r="E13" s="50">
         <f>1.4*E4</f>
         <v/>
       </c>
-      <c r="G13" s="50" t="n"/>
-      <c r="H13" s="45" t="inlineStr">
+      <c r="G13" s="49" t="n"/>
+      <c r="H13" s="44" t="inlineStr">
         <is>
           <t>Pedro</t>
         </is>
       </c>
-      <c r="I13" s="45" t="inlineStr">
+      <c r="I13" s="44" t="inlineStr">
         <is>
           <t>Pleno</t>
         </is>
       </c>
-      <c r="J13" s="141">
+      <c r="J13" s="46">
         <f>VLOOKUP(I13,$A$3:$E$6,5,0)</f>
         <v/>
       </c>
-      <c r="K13" s="141">
+      <c r="K13" s="46">
         <f>VLOOKUP(I13,$A$12:$E$15,5,0)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="50" t="inlineStr">
+      <c r="A14" s="49" t="inlineStr">
         <is>
           <t>Pleno</t>
         </is>
       </c>
-      <c r="B14" s="139">
+      <c r="B14" s="50">
         <f>1.4*B5</f>
         <v/>
       </c>
-      <c r="C14" s="139">
+      <c r="C14" s="50">
         <f>1.4*C5</f>
         <v/>
       </c>
-      <c r="D14" s="139">
+      <c r="D14" s="50">
         <f>1.4*D5</f>
         <v/>
       </c>
-      <c r="E14" s="139">
+      <c r="E14" s="50">
         <f>1.4*E5</f>
         <v/>
       </c>
-      <c r="G14" s="50" t="n"/>
-      <c r="H14" s="45" t="inlineStr">
+      <c r="G14" s="49" t="n"/>
+      <c r="H14" s="44" t="inlineStr">
         <is>
           <t>Diego</t>
         </is>
       </c>
-      <c r="I14" s="45" t="inlineStr">
+      <c r="I14" s="44" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="J14" s="141">
+      <c r="J14" s="46">
         <f>VLOOKUP(I14,$A$3:$E$6,4,0)</f>
         <v/>
       </c>
-      <c r="K14" s="141">
+      <c r="K14" s="46">
         <f>VLOOKUP(I14,$A$12:$E$15,4,0)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="50" t="inlineStr">
+      <c r="A15" s="49" t="inlineStr">
         <is>
           <t>Senior</t>
         </is>
       </c>
-      <c r="B15" s="139">
+      <c r="B15" s="50">
         <f>1.4*B6</f>
         <v/>
       </c>
-      <c r="C15" s="139">
+      <c r="C15" s="50">
         <f>1.4*C6</f>
         <v/>
       </c>
-      <c r="D15" s="139">
+      <c r="D15" s="50">
         <f>1.4*D6</f>
         <v/>
       </c>
-      <c r="E15" s="139">
+      <c r="E15" s="50">
         <f>1.4*E6</f>
         <v/>
       </c>
-      <c r="G15" s="50" t="n"/>
-      <c r="H15" s="45" t="inlineStr">
+      <c r="G15" s="49" t="n"/>
+      <c r="H15" s="44" t="inlineStr">
         <is>
           <t>Leandro</t>
         </is>
       </c>
-      <c r="I15" s="45" t="inlineStr">
+      <c r="I15" s="44" t="inlineStr">
         <is>
           <t>Senior</t>
         </is>
       </c>
-      <c r="J15" s="141">
+      <c r="J15" s="46">
         <f>VLOOKUP(I15,$A$3:$E$6,3,0)</f>
         <v/>
       </c>
-      <c r="K15" s="141">
+      <c r="K15" s="46">
         <f>VLOOKUP(I15,$A$12:$E$15,3,0)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="H16" s="45" t="inlineStr">
+      <c r="H16" s="44" t="inlineStr">
         <is>
           <t>Simas</t>
         </is>
       </c>
-      <c r="I16" s="45" t="inlineStr">
+      <c r="I16" s="44" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="J16" s="141">
+      <c r="J16" s="46">
         <f>VLOOKUP(I16,$A$3:$E$6,3,0)</f>
         <v/>
       </c>
-      <c r="K16" s="141">
+      <c r="K16" s="46">
         <f>VLOOKUP(I16,$A$12:$E$15,3,0)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="H17" s="79" t="inlineStr">
+      <c r="H17" s="77" t="inlineStr">
         <is>
           <t>Alvaro</t>
         </is>
       </c>
-      <c r="I17" s="45" t="inlineStr">
+      <c r="I17" s="44" t="inlineStr">
         <is>
           <t>Estagiário</t>
         </is>
       </c>
-      <c r="J17" s="141">
+      <c r="J17" s="46">
         <f>VLOOKUP(I17,$A$3:$E$6,3,0)</f>
         <v/>
       </c>
-      <c r="K17" s="141">
+      <c r="K17" s="46">
         <f>VLOOKUP(I17,$A$12:$E$15,3,0)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="115" t="inlineStr">
+      <c r="A18" s="113" t="inlineStr">
         <is>
           <t>Consultores Externos</t>
         </is>
       </c>
-      <c r="H18" s="45" t="inlineStr">
+      <c r="H18" s="44" t="inlineStr">
         <is>
           <t>Burato</t>
         </is>
       </c>
-      <c r="I18" s="45" t="inlineStr">
+      <c r="I18" s="44" t="inlineStr">
         <is>
           <t>Externo</t>
         </is>
       </c>
-      <c r="J18" s="141" t="n">
+      <c r="J18" s="46" t="n">
         <v>150</v>
       </c>
-      <c r="K18" s="141" t="n">
+      <c r="K18" s="46" t="n">
         <v>150</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="46" t="inlineStr">
+      <c r="A19" s="45" t="inlineStr">
         <is>
           <t>Carlos Burato</t>
         </is>
       </c>
-      <c r="B19" s="141" t="n">
+      <c r="B19" s="46" t="n">
         <v>150</v>
       </c>
-      <c r="H19" s="45" t="inlineStr">
+      <c r="H19" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">Marcio </t>
         </is>
       </c>
-      <c r="I19" s="45" t="inlineStr">
+      <c r="I19" s="44" t="inlineStr">
         <is>
           <t>Externo</t>
         </is>
       </c>
-      <c r="J19" s="141" t="n">
+      <c r="J19" s="46" t="n">
         <v>100</v>
       </c>
-      <c r="K19" s="141" t="n">
+      <c r="K19" s="46" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="46" t="inlineStr">
+      <c r="A20" s="45" t="inlineStr">
         <is>
           <t>Marcelo Guerra</t>
         </is>
       </c>
-      <c r="B20" s="141" t="n">
+      <c r="B20" s="46" t="n">
         <v>120</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="46" t="inlineStr">
+      <c r="A21" s="45" t="inlineStr">
         <is>
           <t>Marcio Demétrio</t>
         </is>
       </c>
-      <c r="B21" s="141" t="n">
+      <c r="B21" s="46" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>